<commit_message>
Details: cover all Dating & Romance words (81 more, 151 total)
- Nuance/usage (+culture where useful) in 5 languages for every Dating word except 불소
- New tags: romance, drama
- Fix 곰신 (고무신, not 'bear') and 짝남/짝녀 (짝사랑) meanings; mark Verified

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$656</definedName>
@@ -60427,27 +60427,27 @@
       </c>
       <c r="F616" s="16" t="inlineStr">
         <is>
-          <t>Short for "paired-off guy" — the guy someone has a crush on.</t>
+          <t>Short for 짝사랑하는 남자 ("the guy I have a one-sided crush on") — your crush.</t>
         </is>
       </c>
       <c r="G616" s="16" t="inlineStr">
         <is>
-          <t>Abreviatura de "chico emparejado": el chico del que alguien está enamorado.</t>
+          <t>Abreviatura de 짝사랑하는 남자 ("el chico del que estoy enamorada en secreto"): tu crush.</t>
         </is>
       </c>
       <c r="H616" s="16" t="inlineStr">
         <is>
-          <t>「配對男」的簡稱——某人暗戀、有好感的男生。</t>
+          <t>짝사랑하는 남자（暗戀的男生）的縮寫——你暗戀的對象。</t>
         </is>
       </c>
       <c r="I616" s="16" t="inlineStr">
         <is>
-          <t>“配对男”的简称——某人暗恋、有好感的男生。</t>
+          <t>짝사랑하는 남자（暗恋的男生）的缩写——你暗恋的对象。</t>
         </is>
       </c>
       <c r="J616" s="16" t="inlineStr">
         <is>
-          <t>「相手の男」の略——誰かが片思いしている男性。</t>
+          <t>짝사랑하는 남자（片思いしている男性）の略——片思いの相手。</t>
         </is>
       </c>
       <c r="K616" s="16" t="inlineStr">
@@ -60487,7 +60487,7 @@
       </c>
       <c r="R616" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S616" s="15" t="inlineStr">
@@ -60524,27 +60524,27 @@
       </c>
       <c r="F617" s="16" t="inlineStr">
         <is>
-          <t>Short for "paired-off girl" — the girl someone has a crush on.</t>
+          <t>Short for 짝사랑하는 여자 ("the girl I have a one-sided crush on") — your crush.</t>
         </is>
       </c>
       <c r="G617" s="16" t="inlineStr">
         <is>
-          <t>Abreviatura de "chica emparejada": la chica de la que alguien está enamorado.</t>
+          <t>Abreviatura de 짝사랑하는 여자 ("la chica de la que estoy enamorado en secreto"): tu crush.</t>
         </is>
       </c>
       <c r="H617" s="16" t="inlineStr">
         <is>
-          <t>「配對女」的簡稱——某人暗戀、有好感的女生。</t>
+          <t>짝사랑하는 여자（暗戀的女生）的縮寫——你暗戀的對象。</t>
         </is>
       </c>
       <c r="I617" s="16" t="inlineStr">
         <is>
-          <t>“配对女”的简称——某人暗恋、有好感的女生。</t>
+          <t>짝사랑하는 여자（暗恋的女生）的缩写——你暗恋的对象。</t>
         </is>
       </c>
       <c r="J617" s="16" t="inlineStr">
         <is>
-          <t>「相手の女」の略——誰かが片思いしている女性。</t>
+          <t>짝사랑하는 여자（片思いしている女性）の略——片思いの相手。</t>
         </is>
       </c>
       <c r="K617" s="16" t="inlineStr">
@@ -60584,7 +60584,7 @@
       </c>
       <c r="R617" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S617" s="15" t="inlineStr">
@@ -61106,27 +61106,27 @@
       </c>
       <c r="F623" s="16" t="inlineStr">
         <is>
-          <t>"Bear + girlfriend," a term for a girlfriend patiently waiting for her boyfriend to complete mandatory military service.</t>
+          <t>Short for 고무신 (traditional rubber shoes) — a girlfriend patiently waiting for her boyfriend to finish mandatory military service.</t>
         </is>
       </c>
       <c r="G623" s="16" t="inlineStr">
         <is>
-          <t>"Oso + novia", un término para una novia que espera pacientemente a que su novio complete el servicio militar obligatorio.</t>
+          <t>Abreviatura de 고무신 (zapatos tradicionales de goma): una novia que espera pacientemente a que su novio termine el servicio militar obligatorio.</t>
         </is>
       </c>
       <c r="H623" s="16" t="inlineStr">
         <is>
-          <t>「熊＋女友」——耐心等待男友服完兵役的女友暱稱。</t>
+          <t>고무신（傳統膠鞋）的縮寫——耐心等待男友服完兵役的女友。</t>
         </is>
       </c>
       <c r="I623" s="16" t="inlineStr">
         <is>
-          <t>“熊＋女友”——耐心等待男友服完兵役的女友暱称。</t>
+          <t>고무신（传统胶鞋）的缩写——耐心等待男友服完兵役的女友。</t>
         </is>
       </c>
       <c r="J623" s="16" t="inlineStr">
         <is>
-          <t>「熊＋彼女」——兵役を終えるのを我慢強く待つ彼女を指す言葉。</t>
+          <t>고무신（伝統的なゴム靴）の略——兵役を終えるのを待つ彼女のこと。</t>
         </is>
       </c>
       <c r="K623" s="16" t="inlineStr">
@@ -61146,17 +61146,17 @@
       </c>
       <c r="N623" s="16" t="inlineStr">
         <is>
-          <t>熊女友生活還剩六個月了。</t>
+          <t>等男友退伍的日子只剩六個月了。</t>
         </is>
       </c>
       <c r="O623" s="16" t="inlineStr">
         <is>
-          <t>熊女友生活还剩六个月了。</t>
+          <t>等男友退伍的日子只剩六个月了。</t>
         </is>
       </c>
       <c r="P623" s="16" t="inlineStr">
         <is>
-          <t>熊彼女生活、あと6ヶ月残ってる。</t>
+          <t>彼の除隊を待つ生活も、あと6ヶ月。</t>
         </is>
       </c>
       <c r="Q623" s="16" t="inlineStr">
@@ -61166,7 +61166,7 @@
       </c>
       <c r="R623" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S623" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Idol Essentials details (140), Dating guide, remove 불소
- Details for every Idol Essentials word except 사이트석 (term unverified)
- New guide: Korean Dating Slang (36 words, 5 sections)
- Remove unverifiable 불소 (word page deleted)
- Fix 공방 = 공개방송 (music show taping), source: TenAsia 2014; mark Verified
- New tags: industry, stage, beauty

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$656</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$655</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S656"/>
+  <dimension ref="A1:S655"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8144,67 +8144,67 @@
       </c>
       <c r="F77" s="8" t="inlineStr">
         <is>
-          <t>"Public broadcast" — a casual, personal livestream an idol does directly for fans.</t>
+          <t>Short for 공개방송 ("open broadcast") — going in person to a music show's pre-recording or live broadcast to watch and cheer for your idol.</t>
         </is>
       </c>
       <c r="G77" s="8" t="inlineStr">
         <is>
-          <t>"Transmisión pública": una transmisión en vivo casual y personal que un ídolo hace directamente para los fans.</t>
+          <t>Abreviatura de 공개방송 ("emisión abierta"): ir en persona a la pregrabación o la emisión en vivo de un programa musical para ver y animar a tu idol.</t>
         </is>
       </c>
       <c r="H77" s="8" t="inlineStr">
         <is>
-          <t>「公開放送」——偶像直接為粉絲進行的輕鬆個人直播。</t>
+          <t>공개방송（公開放送）的縮寫——親自到音樂節目的事前錄影或直播現場，為偶像應援。</t>
         </is>
       </c>
       <c r="I77" s="8" t="inlineStr">
         <is>
-          <t>“公开放送”——偶像直接为粉丝进行的轻松个人直播。</t>
+          <t>공개방송（公开放送）的缩写——亲自到音乐节目的预录或直播现场，为偶像应援。</t>
         </is>
       </c>
       <c r="J77" s="8" t="inlineStr">
         <is>
-          <t>「公開放送」の略——アイドルがファンのために直接行う気軽な個人配信。</t>
+          <t>공개방송（公開放送）の略——音楽番組の事前収録や生放送の現場に直接行って、推しを応援すること。</t>
         </is>
       </c>
       <c r="K77" s="8" t="inlineStr">
         <is>
-          <t>갑자기 공방 켰어, 빨리 들어가!</t>
+          <t>이번 주 음방 공방 당첨됐어!</t>
         </is>
       </c>
       <c r="L77" s="8" t="inlineStr">
         <is>
-          <t>They suddenly started a livestream, get in quick!</t>
+          <t>I got picked to attend this week's music show taping!</t>
         </is>
       </c>
       <c r="M77" s="8" t="inlineStr">
         <is>
-          <t>¡De repente empezó una transmisión en vivo, entra rápido!</t>
+          <t>¡Me eligieron para ir a la grabación del programa musical de esta semana!</t>
         </is>
       </c>
       <c r="N77" s="8" t="inlineStr">
         <is>
-          <t>突然開了個人直播，快進去！</t>
+          <t>這週音樂節目的公開放送我抽中了！</t>
         </is>
       </c>
       <c r="O77" s="8" t="inlineStr">
         <is>
-          <t>突然开了个人直播，快进去！</t>
+          <t>这周音乐节目的公开放送我抽中了！</t>
         </is>
       </c>
       <c r="P77" s="8" t="inlineStr">
         <is>
-          <t>突然配信始めた、早く入って！</t>
+          <t>今週の音楽番組の公開放送、当選した！</t>
         </is>
       </c>
       <c r="Q77" s="8" t="inlineStr">
         <is>
-          <t>Livestreaming platforms</t>
+          <t>Music show fan culture</t>
         </is>
       </c>
       <c r="R77" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S77" s="7" t="inlineStr">
@@ -64190,12 +64190,12 @@
       </c>
       <c r="B655" s="15" t="inlineStr">
         <is>
-          <t>불소</t>
+          <t>패완얼</t>
         </is>
       </c>
       <c r="C655" s="15" t="inlineStr">
         <is>
-          <t>bul-so</t>
+          <t>pae-wan-eol</t>
         </is>
       </c>
       <c r="D655" s="15" t="inlineStr">
@@ -64210,62 +64210,62 @@
       </c>
       <c r="F655" s="16" t="inlineStr">
         <is>
-          <t>"Burning blind date" — a blind date with intense, immediate chemistry or spark.</t>
+          <t>Short for "fashion is completed by the face" — a saying that a good-looking face elevates any outfit, no matter how simple.</t>
         </is>
       </c>
       <c r="G655" s="16" t="inlineStr">
         <is>
-          <t>"Cita a ciegas ardiente": una cita a ciegas con química o chispa intensa e inmediata.</t>
+          <t>Abreviatura de "la moda se completa con la cara": un dicho que dice que una cara atractiva mejora cualquier atuendo, sin importar lo simple que sea.</t>
         </is>
       </c>
       <c r="H655" s="16" t="inlineStr">
         <is>
-          <t>「燃燒的相親」——雙方一見面就火花四射、氣氛熱烈的相親。</t>
+          <t>「時尚的完成是臉」的簡稱——意指帥氣或漂亮的長相能撐起任何穿搭。</t>
         </is>
       </c>
       <c r="I655" s="16" t="inlineStr">
         <is>
-          <t>“燃烧的相亲”——双方一见面就火花四射、气氛热烈的相亲。</t>
+          <t>“时尚的完成是脸”的简称——意指帅气或漂亮的长相能撑起任何穿搭。</t>
         </is>
       </c>
       <c r="J655" s="16" t="inlineStr">
         <is>
-          <t>「燃える合コン」——一瞬で強い相性や火花が生まれる合コン。</t>
+          <t>「ファッションの完成は顔」の略——どんなにシンプルな服でも、整った顔立ちが引き立てるという言葉。</t>
         </is>
       </c>
       <c r="K655" s="16" t="inlineStr">
         <is>
-          <t>이번 주 불소 잡혔다는데 기대돼.</t>
+          <t>역시 패완얼이야, 뭘 입어도 잘 어울려.</t>
         </is>
       </c>
       <c r="L655" s="16" t="inlineStr">
         <is>
-          <t>I heard there's a fiery blind date lined up this week, I'm excited.</t>
+          <t>It's true, fashion's finished by the face — they look good in anything.</t>
         </is>
       </c>
       <c r="M655" s="16" t="inlineStr">
         <is>
-          <t>Escuché que hay una cita a ciegas con mucha química esta semana, estoy emocionada.</t>
+          <t>Es cierto, la cara lo completa todo — se le ve bien cualquier cosa.</t>
         </is>
       </c>
       <c r="N655" s="16" t="inlineStr">
         <is>
-          <t>聽說這禮拜安排了火花四射的相親，好期待。</t>
+          <t>果然臉才是關鍵，穿什麼都好看。</t>
         </is>
       </c>
       <c r="O655" s="16" t="inlineStr">
         <is>
-          <t>听说这礼拜安排了火花四射的相亲，好期待。</t>
+          <t>果然脸才是关键，穿什么都好看。</t>
         </is>
       </c>
       <c r="P655" s="16" t="inlineStr">
         <is>
-          <t>今週火花散る合コンがセッティングされたって、楽しみ。</t>
+          <t>やっぱり顔が全て、何着ても似合う。</t>
         </is>
       </c>
       <c r="Q655" s="16" t="inlineStr">
         <is>
-          <t>Casual dating talk</t>
+          <t>Fashion/beauty banter</t>
         </is>
       </c>
       <c r="R655" s="15" t="inlineStr">
@@ -64279,105 +64279,8 @@
         </is>
       </c>
     </row>
-    <row r="656" ht="46" customHeight="1">
-      <c r="A656" s="15" t="inlineStr">
-        <is>
-          <t>DAT-082</t>
-        </is>
-      </c>
-      <c r="B656" s="15" t="inlineStr">
-        <is>
-          <t>패완얼</t>
-        </is>
-      </c>
-      <c r="C656" s="15" t="inlineStr">
-        <is>
-          <t>pae-wan-eol</t>
-        </is>
-      </c>
-      <c r="D656" s="15" t="inlineStr">
-        <is>
-          <t>연애 · 썸 표현</t>
-        </is>
-      </c>
-      <c r="E656" s="15" t="inlineStr">
-        <is>
-          <t>Dating &amp; Romance</t>
-        </is>
-      </c>
-      <c r="F656" s="16" t="inlineStr">
-        <is>
-          <t>Short for "fashion is completed by the face" — a saying that a good-looking face elevates any outfit, no matter how simple.</t>
-        </is>
-      </c>
-      <c r="G656" s="16" t="inlineStr">
-        <is>
-          <t>Abreviatura de "la moda se completa con la cara": un dicho que dice que una cara atractiva mejora cualquier atuendo, sin importar lo simple que sea.</t>
-        </is>
-      </c>
-      <c r="H656" s="16" t="inlineStr">
-        <is>
-          <t>「時尚的完成是臉」的簡稱——意指帥氣或漂亮的長相能撐起任何穿搭。</t>
-        </is>
-      </c>
-      <c r="I656" s="16" t="inlineStr">
-        <is>
-          <t>“时尚的完成是脸”的简称——意指帅气或漂亮的长相能撑起任何穿搭。</t>
-        </is>
-      </c>
-      <c r="J656" s="16" t="inlineStr">
-        <is>
-          <t>「ファッションの完成は顔」の略——どんなにシンプルな服でも、整った顔立ちが引き立てるという言葉。</t>
-        </is>
-      </c>
-      <c r="K656" s="16" t="inlineStr">
-        <is>
-          <t>역시 패완얼이야, 뭘 입어도 잘 어울려.</t>
-        </is>
-      </c>
-      <c r="L656" s="16" t="inlineStr">
-        <is>
-          <t>It's true, fashion's finished by the face — they look good in anything.</t>
-        </is>
-      </c>
-      <c r="M656" s="16" t="inlineStr">
-        <is>
-          <t>Es cierto, la cara lo completa todo — se le ve bien cualquier cosa.</t>
-        </is>
-      </c>
-      <c r="N656" s="16" t="inlineStr">
-        <is>
-          <t>果然臉才是關鍵，穿什麼都好看。</t>
-        </is>
-      </c>
-      <c r="O656" s="16" t="inlineStr">
-        <is>
-          <t>果然脸才是关键，穿什么都好看。</t>
-        </is>
-      </c>
-      <c r="P656" s="16" t="inlineStr">
-        <is>
-          <t>やっぱり顔が全て、何着ても似合う。</t>
-        </is>
-      </c>
-      <c r="Q656" s="16" t="inlineStr">
-        <is>
-          <t>Fashion/beauty banter</t>
-        </is>
-      </c>
-      <c r="R656" s="15" t="inlineStr">
-        <is>
-          <t>Draft — please double-check</t>
-        </is>
-      </c>
-      <c r="S656" s="15" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:S656"/>
+  <autoFilter ref="A1:S655"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Nav: add Guides and Quiz to every page; rename 사이트석 → 사이드석
- Guides + Quiz links in desktop nav and mobile menu (all static pages and generators), active state on guide/quiz pages
- Header row widened to 1400px; badge hides at 1360px, hamburger at 1260px (no overflow in any language)
- 사이트석 → 사이드석 (new URL), old URL kept as a noindex redirect; details added

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$655</definedName>
@@ -11422,12 +11422,12 @@
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>사이트석</t>
+          <t>사이드석</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>sa-i-teu-seok</t>
+          <t>sa-i-deu-seok</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
@@ -11467,7 +11467,7 @@
       </c>
       <c r="K111" s="8" t="inlineStr">
         <is>
-          <t>사이트석이라 무대 반쪽만 보였어.</t>
+          <t>사이드석이라 무대 반쪽만 보였어.</t>
         </is>
       </c>
       <c r="L111" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Details: Fandom Feels words (93 more, 509 total); fix 럽콜
- Nuance/usage (+culture where useful) in 5 languages
- 망고주스 sourced (Careet, 2025-08-27)
- 럽콜 meaning fixed to 러브콜 (offer/invitation) in all languages; removes an unfortunate zh-CN example
- Skipped 배댓, 국내반, 해외반 (meanings unverified)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$655</definedName>
@@ -25216,62 +25216,62 @@
       </c>
       <c r="F253" s="10" t="inlineStr">
         <is>
-          <t>"Love call" — an idol affectionately reaching out or calling out to fans during a broadcast.</t>
+          <t>Short for 러브콜 ("love call") — openly saying you want to work with, meet or invite someone: a casting offer, a collab wish, or fans begging for an appearance.</t>
         </is>
       </c>
       <c r="G253" s="10" t="inlineStr">
         <is>
-          <t>"Llamada de amor": un ídolo que se dirige o llama afectuosamente a los fans durante una transmisión.</t>
+          <t>Abreviatura de 러브콜 ("llamada de amor"): decir abiertamente que quieres trabajar con alguien, conocerlo o invitarlo; una oferta de casting, un deseo de colaborar o fans pidiendo una aparición.</t>
         </is>
       </c>
       <c r="H253" s="10" t="inlineStr">
         <is>
-          <t>「愛的呼喚」——偶像在直播中親切地呼喚、招呼粉絲。</t>
+          <t>러브콜（Love call）的縮寫——公開表達想合作、想見面或想邀請某人：選角邀約、合作意願，或粉絲喊話要求上節目。</t>
         </is>
       </c>
       <c r="I253" s="10" t="inlineStr">
         <is>
-          <t>“爱的呼唤”——偶像在直播中亲切地呼唤、招呼粉丝。</t>
+          <t>러브콜（Love call）的缩写——公开表达想合作、想见面或想邀请某人：选角邀约、合作意愿，或粉丝喊话要求上节目。</t>
         </is>
       </c>
       <c r="J253" s="10" t="inlineStr">
         <is>
-          <t>「愛の呼びかけ」——配信中にアイドルが愛情を込めてファンに呼びかけること。</t>
+          <t>러브콜（ラブコール）の略——一緒に仕事したい、会いたい、招きたいと公に伝えること。キャスティングのオファー、コラボの希望、ファンの出演リクエストなど。</t>
         </is>
       </c>
       <c r="K253" s="10" t="inlineStr">
         <is>
-          <t>럽콜 해줄 때마다 심장 터질 것 같아.</t>
+          <t>그 예능에서 계속 럽콜 보내는 중이래.</t>
         </is>
       </c>
       <c r="L253" s="10" t="inlineStr">
         <is>
-          <t>My heart feels like it'll burst every time they do a love call.</t>
+          <t>I heard that variety show keeps sending her love calls to appear.</t>
         </is>
       </c>
       <c r="M253" s="10" t="inlineStr">
         <is>
-          <t>Siento que mi corazón va a estallar cada vez que hace una llamada de cariño.</t>
+          <t>Dicen que ese programa de variedades no deja de invitarla.</t>
         </is>
       </c>
       <c r="N253" s="10" t="inlineStr">
         <is>
-          <t>每次做愛的呼喚我的心都要跳出來了。</t>
+          <t>聽說那個綜藝一直向她發出邀約。</t>
         </is>
       </c>
       <c r="O253" s="10" t="inlineStr">
         <is>
-          <t>每次做爱的呼唤我的心都要跳出来了。</t>
+          <t>听说那个综艺一直向她发出邀约。</t>
         </is>
       </c>
       <c r="P253" s="10" t="inlineStr">
         <is>
-          <t>ラブコールしてくれるたびに、心臓が爆発しそう。</t>
+          <t>あのバラエティ番組がずっと彼女にラブコールを送ってるらしい。</t>
         </is>
       </c>
       <c r="Q253" s="10" t="inlineStr">
         <is>
-          <t>Livestream fan reactions</t>
+          <t>Collab and casting news</t>
         </is>
       </c>
       <c r="R253" s="9" t="inlineStr">
@@ -26726,7 +26726,7 @@
       </c>
       <c r="Q268" s="10" t="inlineStr">
         <is>
-          <t>K-pop fan messaging app culture, 2026 slang</t>
+          <t>K-pop fan messaging app culture, 2025 meme</t>
         </is>
       </c>
       <c r="R268" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Fix 배댓 → 베댓 (best comment), 국내반/해외반 = album editions
- Meanings rewritten in all 5 languages, details added
- Old word/bae-daet.html kept as noindex redirect

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$655</definedName>
@@ -17727,12 +17727,12 @@
       </c>
       <c r="B176" s="9" t="inlineStr">
         <is>
-          <t>배댓</t>
+          <t>베댓</t>
         </is>
       </c>
       <c r="C176" s="9" t="inlineStr">
         <is>
-          <t>bae-daet</t>
+          <t>be-daet</t>
         </is>
       </c>
       <c r="D176" s="9" t="inlineStr">
@@ -17747,42 +17747,42 @@
       </c>
       <c r="F176" s="10" t="inlineStr">
         <is>
-          <t>A "belly comment" — a witty first comment posted right under an official account's post.</t>
+          <t>Short for 베스트 댓글 ("best comment"): the top-ranked, most-liked comment shown first under a post or article.</t>
         </is>
       </c>
       <c r="G176" s="10" t="inlineStr">
         <is>
-          <t>Un "comentario de vientre": un comentario ingenioso publicado justo debajo de una publicación de una cuenta oficial.</t>
+          <t>Abreviatura de 베스트 댓글 ("mejor comentario"): el comentario con más likes, que aparece primero bajo una publicación o noticia.</t>
         </is>
       </c>
       <c r="H176" s="10" t="inlineStr">
         <is>
-          <t>「肚子留言」——搶在官方帳號貼文下第一時間發的機智留言。</t>
+          <t>베스트 댓글（最佳留言）的縮寫：貼文或新聞下按讚最多、排在最上面的留言。</t>
         </is>
       </c>
       <c r="I176" s="10" t="inlineStr">
         <is>
-          <t>“肚子留言”——抢在官方帐号贴文下第一时间发的机智留言。</t>
+          <t>베스트 댓글（最佳留言）的缩写：帖子或新闻下点赞最多、排在最上面的留言。</t>
         </is>
       </c>
       <c r="J176" s="10" t="inlineStr">
         <is>
-          <t>公式アカウントの投稿の下に一番乗りで書かれる気の利いたコメント。</t>
+          <t>베스트 댓글（ベストコメント）の略——投稿や記事の下で一番いいねが多く、上に表示されるコメント。</t>
         </is>
       </c>
       <c r="K176" s="10" t="inlineStr">
         <is>
-          <t>배댓 진짜 웃겨서 캡처했어.</t>
+          <t>베댓 진짜 웃겨서 캡처했어.</t>
         </is>
       </c>
       <c r="L176" s="10" t="inlineStr">
         <is>
-          <t>The belly comment was so funny I took a screenshot.</t>
+          <t>The top comment was so funny I took a screenshot.</t>
         </is>
       </c>
       <c r="M176" s="10" t="inlineStr">
         <is>
-          <t>El primer comentario fue tan gracioso que le tomé captura.</t>
+          <t>El comentario destacado fue tan gracioso que le tomé captura.</t>
         </is>
       </c>
       <c r="N176" s="10" t="inlineStr">
@@ -17792,17 +17792,17 @@
       </c>
       <c r="O176" s="10" t="inlineStr">
         <is>
-          <t>那则神留言太好笑了，我截屏了。</t>
+          <t>那条神评论太好笑了，我截屏了。</t>
         </is>
       </c>
       <c r="P176" s="10" t="inlineStr">
         <is>
-          <t>神コメント面白すぎてスクショした。</t>
+          <t>ベストコメントが面白すぎてスクショした。</t>
         </is>
       </c>
       <c r="Q176" s="10" t="inlineStr">
         <is>
-          <t>Official social posts</t>
+          <t>Comment sections</t>
         </is>
       </c>
       <c r="R176" s="9" t="inlineStr">
@@ -22015,62 +22015,62 @@
       </c>
       <c r="F220" s="10" t="inlineStr">
         <is>
-          <t>"Domestic half" — the portion of a fandom based within Korea, as opposed to overseas.</t>
+          <t>국내 + 盤 ("record, edition"): the Korean domestic release of an album, as opposed to overseas editions like the Japanese one.</t>
         </is>
       </c>
       <c r="G220" s="10" t="inlineStr">
         <is>
-          <t>"Mitad doméstica": la parte del fandom que reside dentro de Corea, en contraste con el extranjero.</t>
+          <t>국내 + 盤 ("disco, edición"): la edición coreana nacional de un álbum, frente a las ediciones extranjeras como la japonesa.</t>
         </is>
       </c>
       <c r="H220" s="10" t="inlineStr">
         <is>
-          <t>「國內組」——粉絲圈中位於韓國國內的部分，相對於海外組。</t>
+          <t>國內盤——專輯在韓國國內發行的版本，相對於日本盤等海外版本。</t>
         </is>
       </c>
       <c r="I220" s="10" t="inlineStr">
         <is>
-          <t>“国内组”——粉丝圈中位于韩国国内的部分，相对于海外组。</t>
+          <t>国内盘——专辑在韩国国内发行的版本，相对于日本盘等海外版本。</t>
         </is>
       </c>
       <c r="J220" s="10" t="inlineStr">
         <is>
-          <t>「国内組」——海外ではなく、韓国国内を拠点とするファンダムの部分。</t>
+          <t>国内盤——アルバムの韓国国内リリース版。日本盤など海外版との対比で使う。</t>
         </is>
       </c>
       <c r="K220" s="10" t="inlineStr">
         <is>
-          <t>국내반이랑 해외반이랑 반응이 다르네.</t>
+          <t>국내반이랑 일본반 구성이 달라.</t>
         </is>
       </c>
       <c r="L220" s="10" t="inlineStr">
         <is>
-          <t>The domestic and overseas fandoms are reacting differently.</t>
+          <t>The Korean edition and the Japanese edition have different contents.</t>
         </is>
       </c>
       <c r="M220" s="10" t="inlineStr">
         <is>
-          <t>El fandom nacional y el internacional están reaccionando distinto.</t>
+          <t>La edición coreana y la japonesa traen contenidos distintos.</t>
         </is>
       </c>
       <c r="N220" s="10" t="inlineStr">
         <is>
-          <t>國內飯跟海外飯反應不太一樣。</t>
+          <t>韓國盤和日本盤的內容不一樣。</t>
         </is>
       </c>
       <c r="O220" s="10" t="inlineStr">
         <is>
-          <t>国内饭跟海外饭反应不太一样。</t>
+          <t>韩国盘和日本盘的内容不一样。</t>
         </is>
       </c>
       <c r="P220" s="10" t="inlineStr">
         <is>
-          <t>国内担と海外担で反応が違うね。</t>
+          <t>韓国盤と日本盤は構成が違う。</t>
         </is>
       </c>
       <c r="Q220" s="10" t="inlineStr">
         <is>
-          <t>Fandom comparison talk</t>
+          <t>Album collecting talk</t>
         </is>
       </c>
       <c r="R220" s="9" t="inlineStr">
@@ -22112,62 +22112,62 @@
       </c>
       <c r="F221" s="10" t="inlineStr">
         <is>
-          <t>"Overseas half" — the portion of a fandom based outside Korea.</t>
+          <t>해외 + 盤 ("record, edition"): an album version released outside Korea — such as a Japanese or US edition — often with different photos, photocards or tracks.</t>
         </is>
       </c>
       <c r="G221" s="10" t="inlineStr">
         <is>
-          <t>"Mitad extranjera": la parte del fandom que reside fuera de Corea.</t>
+          <t>해외 + 盤 ("disco, edición"): una versión del álbum lanzada fuera de Corea, como la edición japonesa o estadounidense, a menudo con fotos, photocards o canciones distintas.</t>
         </is>
       </c>
       <c r="H221" s="10" t="inlineStr">
         <is>
-          <t>「海外組」——粉絲圈中位於韓國以外地區的部分。</t>
+          <t>海外盤——在韓國以外發行的專輯版本（如日本盤、美國版），照片、小卡或收錄曲常不同。</t>
         </is>
       </c>
       <c r="I221" s="10" t="inlineStr">
         <is>
-          <t>“海外组”——粉丝圈中位于韩国以外地区的部分。</t>
+          <t>海外盘——在韩国以外发行的专辑版本（如日本盘、美国版），照片、小卡或收录曲常不同。</t>
         </is>
       </c>
       <c r="J221" s="10" t="inlineStr">
         <is>
-          <t>「海外組」——韓国以外を拠点とするファンダムの部分。</t>
+          <t>海外盤——韓国以外でリリースされるアルバムの版（日本盤や米国盤など）。写真やトレカ、収録曲が違うことも多い。</t>
         </is>
       </c>
       <c r="K221" s="10" t="inlineStr">
         <is>
-          <t>해외반이 스밍을 진짜 열심히 해.</t>
+          <t>해외반에만 들어 있는 포카가 따로 있대.</t>
         </is>
       </c>
       <c r="L221" s="10" t="inlineStr">
         <is>
-          <t>The overseas fandom streams really hard.</t>
+          <t>I heard there are photocards that only come in the overseas edition.</t>
         </is>
       </c>
       <c r="M221" s="10" t="inlineStr">
         <is>
-          <t>El fandom internacional hace streaming con muchísimo esfuerzo.</t>
+          <t>Dicen que hay photocards que solo vienen en la edición internacional.</t>
         </is>
       </c>
       <c r="N221" s="10" t="inlineStr">
         <is>
-          <t>海外飯刷榜真的很認真。</t>
+          <t>聽說有只放在海外盤裡的小卡。</t>
         </is>
       </c>
       <c r="O221" s="10" t="inlineStr">
         <is>
-          <t>海外饭刷榜真的很认真。</t>
+          <t>听说有只放在海外盘里的小卡。</t>
         </is>
       </c>
       <c r="P221" s="10" t="inlineStr">
         <is>
-          <t>海外担のストリーミング、本当に頑張ってる。</t>
+          <t>海外盤にしか入っていないトレカがあるらしい。</t>
         </is>
       </c>
       <c r="Q221" s="10" t="inlineStr">
         <is>
-          <t>Fandom comparison talk</t>
+          <t>Album collecting talk</t>
         </is>
       </c>
       <c r="R221" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Details: Online Memes (142) — every word now has details (654/654)
- Nuance/usage (+culture where useful) in 5 languages
- Fix 혜자스럽다 origin (Kim Hye-ja lunch box, 2010; Maeil Shinmun 2023) and mark Verified
- Usage caveats for 오또케, 오조오억, 샤갈 instead of invented origins
- New tags: worklife, food; CLAUDE.md notes details are complete

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$655</definedName>
@@ -45780,27 +45780,27 @@
       </c>
       <c r="F465" s="14" t="inlineStr">
         <is>
-          <t>"Hyeja-like" — describes a generous portion or great value, named after a historical figure known for generosity.</t>
+          <t>"Hyeja-like" — generous portions or great value for the price. It comes from a convenience-store lunch box launched in 2010 with actress Kim Hye-ja, famous for packing a lot in for little money.</t>
         </is>
       </c>
       <c r="G465" s="14" t="inlineStr">
         <is>
-          <t>"Como Hyeja": describe una porción generosa o un gran valor, en honor a una figura histórica conocida por su generosidad.</t>
+          <t>"Como Hyeja": porciones generosas o gran relación calidad-precio. Viene de una lonchera de tienda de conveniencia lanzada en 2010 con la actriz Kim Hye-ja, famosa por traer mucho por poco dinero.</t>
         </is>
       </c>
       <c r="H465" s="14" t="inlineStr">
         <is>
-          <t>「惠子式的」——形容份量大方、CP值高，源自一位以慷慨聞名的歷史人物名字。</t>
+          <t>「惠子式的」——形容份量大方、CP值高。源自2010年與演員金惠子合作推出、以便宜又豐盛聞名的便利商店便當。</t>
         </is>
       </c>
       <c r="I465" s="14" t="inlineStr">
         <is>
-          <t>“惠子式的”——形容份量大方、CP值高，源自一位以慷慨闻名的历史人物名字。</t>
+          <t>“惠子式的”——形容份量大方、性价比高。源自2010年与演员金惠子合作推出、以便宜又丰盛闻名的便利店便当。</t>
         </is>
       </c>
       <c r="J465" s="14" t="inlineStr">
         <is>
-          <t>気前が良く、コスパが良いことを表す——寛大さで知られた歴史上の人物の名前から来ている。</t>
+          <t>「ヘジャっぽい」——量が多くてコスパが良いこと。2010年に女優キム・ヘジャさんと発売された、安くてボリューム満点のコンビニ弁当が由来。</t>
         </is>
       </c>
       <c r="K465" s="14" t="inlineStr">
@@ -45825,12 +45825,12 @@
       </c>
       <c r="O465" s="14" t="inlineStr">
         <is>
-          <t>这家餐厅份量真的很佛心。</t>
+          <t>这家餐厅份量真的很良心。</t>
         </is>
       </c>
       <c r="P465" s="14" t="inlineStr">
         <is>
-          <t>このお店、マジで太っ腹だよね。</t>
+          <t>このお店、マジでボリュームたっぷり。</t>
         </is>
       </c>
       <c r="Q465" s="14" t="inlineStr">
@@ -45840,7 +45840,7 @@
       </c>
       <c r="R465" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S465" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Add swear tag and 'Korean Swear Words, Explained' guide
- New 'swear' tag (5 languages) on 20 vulgar/crude-intensifier words
- Guide with 5 sections + per-section strength notes (optional 'note' field in COLLECTIONS)
- 씨발/지랄/미친/젠장/병맛/시발비용 verified with sources (Wikipedia, Kyunghyang, Newsis)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$760</definedName>
@@ -42736,7 +42736,7 @@
       </c>
       <c r="R433" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S433" s="11" t="inlineStr">
@@ -65531,7 +65531,7 @@
       </c>
       <c r="R668" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S668" s="13" t="inlineStr">
@@ -65919,7 +65919,7 @@
       </c>
       <c r="R672" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S672" s="13" t="inlineStr">
@@ -66016,7 +66016,7 @@
       </c>
       <c r="R673" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S673" s="13" t="inlineStr">
@@ -66113,7 +66113,7 @@
       </c>
       <c r="R674" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S674" s="13" t="inlineStr">
@@ -66307,7 +66307,7 @@
       </c>
       <c r="R676" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S676" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Verify 202 Draft words with sources (batch 1)
Each newly Verified word gets the page(s) its meaning was checked against
(news articles, Wikipedia, KoreanClass101, Soompi, Hanteo News, etc.).
Also fixes a typo in 머선129 (일이구 -> 일이고).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$770</definedName>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="R6" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S6" s="7" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S7" s="7" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="R8" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S8" s="7" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="R9" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S9" s="7" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="R20" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S20" s="7" t="inlineStr">
@@ -2869,7 +2869,7 @@
       </c>
       <c r="R22" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S22" s="7" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="R23" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S23" s="7" t="inlineStr">
@@ -3063,7 +3063,7 @@
       </c>
       <c r="R24" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S24" s="7" t="inlineStr">
@@ -3257,7 +3257,7 @@
       </c>
       <c r="R26" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S26" s="7" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="R27" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S27" s="7" t="inlineStr">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="R28" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S28" s="7" t="inlineStr">
@@ -3645,7 +3645,7 @@
       </c>
       <c r="R30" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S30" s="7" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="R36" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S36" s="7" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="R37" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S37" s="7" t="inlineStr">
@@ -4518,7 +4518,7 @@
       </c>
       <c r="R39" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S39" s="7" t="inlineStr">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="R41" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S41" s="7" t="inlineStr">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="R42" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S42" s="7" t="inlineStr">
@@ -6555,7 +6555,7 @@
       </c>
       <c r="R60" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S60" s="7" t="inlineStr">
@@ -6749,7 +6749,7 @@
       </c>
       <c r="R62" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S62" s="7" t="inlineStr">
@@ -6846,7 +6846,7 @@
       </c>
       <c r="R63" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S63" s="7" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="R64" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S64" s="7" t="inlineStr">
@@ -7040,7 +7040,7 @@
       </c>
       <c r="R65" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S65" s="7" t="inlineStr">
@@ -8689,7 +8689,7 @@
       </c>
       <c r="R82" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S82" s="7" t="inlineStr">
@@ -9077,7 +9077,7 @@
       </c>
       <c r="R86" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S86" s="7" t="inlineStr">
@@ -11017,7 +11017,7 @@
       </c>
       <c r="R106" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S106" s="7" t="inlineStr">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="R150" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S150" s="7" t="inlineStr">
@@ -16352,7 +16352,7 @@
       </c>
       <c r="R161" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S161" s="7" t="inlineStr">
@@ -17031,7 +17031,7 @@
       </c>
       <c r="R168" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S168" s="7" t="inlineStr">
@@ -17225,7 +17225,7 @@
       </c>
       <c r="R170" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S170" s="7" t="inlineStr">
@@ -18001,7 +18001,7 @@
       </c>
       <c r="R178" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S178" s="9" t="inlineStr">
@@ -18486,7 +18486,7 @@
       </c>
       <c r="R183" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S183" s="9" t="inlineStr">
@@ -18777,7 +18777,7 @@
       </c>
       <c r="R186" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S186" s="9" t="inlineStr">
@@ -19068,7 +19068,7 @@
       </c>
       <c r="R189" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S189" s="9" t="inlineStr">
@@ -19456,7 +19456,7 @@
       </c>
       <c r="R193" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S193" s="9" t="inlineStr">
@@ -20038,7 +20038,7 @@
       </c>
       <c r="R199" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S199" s="9" t="inlineStr">
@@ -20232,7 +20232,7 @@
       </c>
       <c r="R201" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S201" s="9" t="inlineStr">
@@ -21493,7 +21493,7 @@
       </c>
       <c r="R214" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S214" s="9" t="inlineStr">
@@ -21590,7 +21590,7 @@
       </c>
       <c r="R215" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S215" s="9" t="inlineStr">
@@ -22366,7 +22366,7 @@
       </c>
       <c r="R223" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S223" s="9" t="inlineStr">
@@ -23821,7 +23821,7 @@
       </c>
       <c r="R238" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S238" s="9" t="inlineStr">
@@ -23918,7 +23918,7 @@
       </c>
       <c r="R239" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S239" s="9" t="inlineStr">
@@ -24791,7 +24791,7 @@
       </c>
       <c r="R248" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S248" s="9" t="inlineStr">
@@ -24985,7 +24985,7 @@
       </c>
       <c r="R250" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S250" s="9" t="inlineStr">
@@ -25955,7 +25955,7 @@
       </c>
       <c r="R260" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S260" s="9" t="inlineStr">
@@ -26440,7 +26440,7 @@
       </c>
       <c r="R265" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S265" s="9" t="inlineStr">
@@ -27119,7 +27119,7 @@
       </c>
       <c r="R272" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S272" s="9" t="inlineStr">
@@ -29059,7 +29059,7 @@
       </c>
       <c r="R292" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S292" s="9" t="inlineStr">
@@ -30611,7 +30611,7 @@
       </c>
       <c r="R308" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S308" s="11" t="inlineStr">
@@ -30708,7 +30708,7 @@
       </c>
       <c r="R309" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S309" s="11" t="inlineStr">
@@ -30805,7 +30805,7 @@
       </c>
       <c r="R310" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S310" s="11" t="inlineStr">
@@ -30902,7 +30902,7 @@
       </c>
       <c r="R311" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S311" s="11" t="inlineStr">
@@ -31387,7 +31387,7 @@
       </c>
       <c r="R316" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S316" s="11" t="inlineStr">
@@ -31581,7 +31581,7 @@
       </c>
       <c r="R318" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S318" s="11" t="inlineStr">
@@ -31678,7 +31678,7 @@
       </c>
       <c r="R319" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S319" s="11" t="inlineStr">
@@ -31775,7 +31775,7 @@
       </c>
       <c r="R320" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S320" s="11" t="inlineStr">
@@ -31872,7 +31872,7 @@
       </c>
       <c r="R321" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S321" s="11" t="inlineStr">
@@ -31969,7 +31969,7 @@
       </c>
       <c r="R322" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S322" s="11" t="inlineStr">
@@ -32260,7 +32260,7 @@
       </c>
       <c r="R325" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S325" s="11" t="inlineStr">
@@ -32357,7 +32357,7 @@
       </c>
       <c r="R326" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S326" s="11" t="inlineStr">
@@ -32551,7 +32551,7 @@
       </c>
       <c r="R328" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S328" s="11" t="inlineStr">
@@ -32648,7 +32648,7 @@
       </c>
       <c r="R329" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S329" s="11" t="inlineStr">
@@ -32842,7 +32842,7 @@
       </c>
       <c r="R331" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S331" s="11" t="inlineStr">
@@ -33036,7 +33036,7 @@
       </c>
       <c r="R333" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S333" s="11" t="inlineStr">
@@ -33327,7 +33327,7 @@
       </c>
       <c r="R336" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S336" s="11" t="inlineStr">
@@ -33424,7 +33424,7 @@
       </c>
       <c r="R337" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S337" s="11" t="inlineStr">
@@ -33812,7 +33812,7 @@
       </c>
       <c r="R341" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S341" s="11" t="inlineStr">
@@ -34103,7 +34103,7 @@
       </c>
       <c r="R344" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S344" s="11" t="inlineStr">
@@ -35364,7 +35364,7 @@
       </c>
       <c r="R357" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S357" s="11" t="inlineStr">
@@ -35558,7 +35558,7 @@
       </c>
       <c r="R359" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S359" s="11" t="inlineStr">
@@ -35655,7 +35655,7 @@
       </c>
       <c r="R360" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S360" s="11" t="inlineStr">
@@ -35946,7 +35946,7 @@
       </c>
       <c r="R363" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S363" s="11" t="inlineStr">
@@ -38759,7 +38759,7 @@
       </c>
       <c r="R392" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S392" s="11" t="inlineStr">
@@ -38856,7 +38856,7 @@
       </c>
       <c r="R393" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S393" s="11" t="inlineStr">
@@ -38953,7 +38953,7 @@
       </c>
       <c r="R394" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S394" s="11" t="inlineStr">
@@ -39050,7 +39050,7 @@
       </c>
       <c r="R395" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S395" s="11" t="inlineStr">
@@ -39147,7 +39147,7 @@
       </c>
       <c r="R396" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S396" s="11" t="inlineStr">
@@ -39244,7 +39244,7 @@
       </c>
       <c r="R397" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S397" s="11" t="inlineStr">
@@ -40020,7 +40020,7 @@
       </c>
       <c r="R405" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S405" s="11" t="inlineStr">
@@ -41669,7 +41669,7 @@
       </c>
       <c r="R422" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S422" s="11" t="inlineStr">
@@ -42542,7 +42542,7 @@
       </c>
       <c r="R431" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S431" s="11" t="inlineStr">
@@ -42639,7 +42639,7 @@
       </c>
       <c r="R432" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S432" s="11" t="inlineStr">
@@ -42930,7 +42930,7 @@
       </c>
       <c r="R435" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S435" s="13" t="inlineStr">
@@ -43027,7 +43027,7 @@
       </c>
       <c r="R436" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S436" s="13" t="inlineStr">
@@ -43124,7 +43124,7 @@
       </c>
       <c r="R437" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S437" s="13" t="inlineStr">
@@ -43221,7 +43221,7 @@
       </c>
       <c r="R438" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S438" s="13" t="inlineStr">
@@ -43318,7 +43318,7 @@
       </c>
       <c r="R439" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S439" s="13" t="inlineStr">
@@ -43415,7 +43415,7 @@
       </c>
       <c r="R440" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S440" s="13" t="inlineStr">
@@ -43512,7 +43512,7 @@
       </c>
       <c r="R441" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S441" s="13" t="inlineStr">
@@ -43609,7 +43609,7 @@
       </c>
       <c r="R442" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S442" s="13" t="inlineStr">
@@ -43803,7 +43803,7 @@
       </c>
       <c r="R444" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S444" s="13" t="inlineStr">
@@ -43997,7 +43997,7 @@
       </c>
       <c r="R446" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S446" s="13" t="inlineStr">
@@ -44094,7 +44094,7 @@
       </c>
       <c r="R447" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S447" s="13" t="inlineStr">
@@ -45452,7 +45452,7 @@
       </c>
       <c r="R461" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S461" s="13" t="inlineStr">
@@ -45549,7 +45549,7 @@
       </c>
       <c r="R462" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S462" s="13" t="inlineStr">
@@ -45743,7 +45743,7 @@
       </c>
       <c r="R464" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S464" s="13" t="inlineStr">
@@ -46422,7 +46422,7 @@
       </c>
       <c r="R471" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S471" s="13" t="inlineStr">
@@ -46519,7 +46519,7 @@
       </c>
       <c r="R472" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S472" s="13" t="inlineStr">
@@ -46616,7 +46616,7 @@
       </c>
       <c r="R473" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S473" s="13" t="inlineStr">
@@ -46713,7 +46713,7 @@
       </c>
       <c r="R474" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S474" s="13" t="inlineStr">
@@ -46810,7 +46810,7 @@
       </c>
       <c r="R475" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S475" s="13" t="inlineStr">
@@ -47004,7 +47004,7 @@
       </c>
       <c r="R477" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S477" s="13" t="inlineStr">
@@ -47101,7 +47101,7 @@
       </c>
       <c r="R478" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S478" s="13" t="inlineStr">
@@ -47198,7 +47198,7 @@
       </c>
       <c r="R479" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S479" s="13" t="inlineStr">
@@ -47392,7 +47392,7 @@
       </c>
       <c r="R481" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S481" s="13" t="inlineStr">
@@ -47489,7 +47489,7 @@
       </c>
       <c r="R482" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S482" s="13" t="inlineStr">
@@ -48168,7 +48168,7 @@
       </c>
       <c r="R489" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S489" s="13" t="inlineStr">
@@ -48265,7 +48265,7 @@
       </c>
       <c r="R490" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S490" s="13" t="inlineStr">
@@ -48362,7 +48362,7 @@
       </c>
       <c r="R491" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S491" s="13" t="inlineStr">
@@ -48459,7 +48459,7 @@
       </c>
       <c r="R492" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S492" s="13" t="inlineStr">
@@ -48556,7 +48556,7 @@
       </c>
       <c r="R493" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S493" s="13" t="inlineStr">
@@ -48653,7 +48653,7 @@
       </c>
       <c r="R494" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S494" s="13" t="inlineStr">
@@ -48750,7 +48750,7 @@
       </c>
       <c r="R495" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S495" s="13" t="inlineStr">
@@ -48847,7 +48847,7 @@
       </c>
       <c r="R496" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S496" s="13" t="inlineStr">
@@ -48944,7 +48944,7 @@
       </c>
       <c r="R497" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S497" s="13" t="inlineStr">
@@ -49041,7 +49041,7 @@
       </c>
       <c r="R498" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S498" s="13" t="inlineStr">
@@ -49526,7 +49526,7 @@
       </c>
       <c r="R503" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S503" s="13" t="inlineStr">
@@ -49817,7 +49817,7 @@
       </c>
       <c r="R506" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S506" s="13" t="inlineStr">
@@ -49914,7 +49914,7 @@
       </c>
       <c r="R507" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S507" s="13" t="inlineStr">
@@ -50011,7 +50011,7 @@
       </c>
       <c r="R508" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S508" s="13" t="inlineStr">
@@ -50108,7 +50108,7 @@
       </c>
       <c r="R509" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S509" s="13" t="inlineStr">
@@ -50302,7 +50302,7 @@
       </c>
       <c r="R511" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S511" s="13" t="inlineStr">
@@ -50690,7 +50690,7 @@
       </c>
       <c r="R515" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S515" s="13" t="inlineStr">
@@ -50884,7 +50884,7 @@
       </c>
       <c r="R517" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S517" s="13" t="inlineStr">
@@ -50981,7 +50981,7 @@
       </c>
       <c r="R518" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S518" s="13" t="inlineStr">
@@ -51757,7 +51757,7 @@
       </c>
       <c r="R526" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S526" s="13" t="inlineStr">
@@ -52048,7 +52048,7 @@
       </c>
       <c r="R529" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S529" s="13" t="inlineStr">
@@ -53212,7 +53212,7 @@
       </c>
       <c r="R541" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S541" s="13" t="inlineStr">
@@ -53406,7 +53406,7 @@
       </c>
       <c r="R543" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S543" s="13" t="inlineStr">
@@ -53503,7 +53503,7 @@
       </c>
       <c r="R544" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S544" s="13" t="inlineStr">
@@ -53600,7 +53600,7 @@
       </c>
       <c r="R545" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S545" s="13" t="inlineStr">
@@ -53794,7 +53794,7 @@
       </c>
       <c r="R547" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S547" s="13" t="inlineStr">
@@ -53891,7 +53891,7 @@
       </c>
       <c r="R548" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S548" s="13" t="inlineStr">
@@ -53988,7 +53988,7 @@
       </c>
       <c r="R549" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S549" s="13" t="inlineStr">
@@ -56316,7 +56316,7 @@
       </c>
       <c r="R573" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S573" s="13" t="inlineStr">
@@ -56413,7 +56413,7 @@
       </c>
       <c r="R574" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S574" s="13" t="inlineStr">
@@ -56607,7 +56607,7 @@
       </c>
       <c r="R576" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S576" s="13" t="inlineStr">
@@ -56704,7 +56704,7 @@
       </c>
       <c r="R577" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S577" s="13" t="inlineStr">
@@ -56898,7 +56898,7 @@
       </c>
       <c r="R579" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S579" s="13" t="inlineStr">
@@ -57092,7 +57092,7 @@
       </c>
       <c r="R581" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S581" s="13" t="inlineStr">
@@ -57189,7 +57189,7 @@
       </c>
       <c r="R582" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S582" s="13" t="inlineStr">
@@ -57286,7 +57286,7 @@
       </c>
       <c r="R583" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S583" s="13" t="inlineStr">
@@ -57868,7 +57868,7 @@
       </c>
       <c r="R589" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S589" s="13" t="inlineStr">
@@ -57965,7 +57965,7 @@
       </c>
       <c r="R590" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S590" s="13" t="inlineStr">
@@ -58256,7 +58256,7 @@
       </c>
       <c r="R593" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S593" s="13" t="inlineStr">
@@ -59420,7 +59420,7 @@
       </c>
       <c r="R605" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S605" s="13" t="inlineStr">
@@ -59517,7 +59517,7 @@
       </c>
       <c r="R606" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S606" s="13" t="inlineStr">
@@ -59808,7 +59808,7 @@
       </c>
       <c r="R609" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S609" s="13" t="inlineStr">
@@ -59905,7 +59905,7 @@
       </c>
       <c r="R610" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S610" s="13" t="inlineStr">
@@ -60002,7 +60002,7 @@
       </c>
       <c r="R611" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S611" s="13" t="inlineStr">
@@ -60390,7 +60390,7 @@
       </c>
       <c r="R615" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S615" s="13" t="inlineStr">
@@ -60584,7 +60584,7 @@
       </c>
       <c r="R617" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S617" s="13" t="inlineStr">
@@ -60875,7 +60875,7 @@
       </c>
       <c r="R620" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S620" s="13" t="inlineStr">
@@ -61166,7 +61166,7 @@
       </c>
       <c r="R623" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S623" s="13" t="inlineStr">
@@ -61203,7 +61203,7 @@
       </c>
       <c r="F624" s="14" t="inlineStr">
         <is>
-          <t>A dialect-flavored "what's going on?" (무슨 일이고) where 일이구 is written as the numbers 129.</t>
+          <t>A dialect-flavored "what's going on?" (무슨 일이고) where 일이고 is written as the numbers 129.</t>
         </is>
       </c>
       <c r="G624" s="14" t="inlineStr">
@@ -61360,7 +61360,7 @@
       </c>
       <c r="R625" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S625" s="13" t="inlineStr">
@@ -61457,7 +61457,7 @@
       </c>
       <c r="R626" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S626" s="13" t="inlineStr">
@@ -61748,7 +61748,7 @@
       </c>
       <c r="R629" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S629" s="13" t="inlineStr">
@@ -61942,7 +61942,7 @@
       </c>
       <c r="R631" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S631" s="13" t="inlineStr">
@@ -62136,7 +62136,7 @@
       </c>
       <c r="R633" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S633" s="13" t="inlineStr">
@@ -62233,7 +62233,7 @@
       </c>
       <c r="R634" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S634" s="13" t="inlineStr">
@@ -62330,7 +62330,7 @@
       </c>
       <c r="R635" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S635" s="13" t="inlineStr">
@@ -62524,7 +62524,7 @@
       </c>
       <c r="R637" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S637" s="13" t="inlineStr">
@@ -62718,7 +62718,7 @@
       </c>
       <c r="R639" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S639" s="13" t="inlineStr">
@@ -62815,7 +62815,7 @@
       </c>
       <c r="R640" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S640" s="13" t="inlineStr">
@@ -63203,7 +63203,7 @@
       </c>
       <c r="R644" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S644" s="13" t="inlineStr">
@@ -63397,7 +63397,7 @@
       </c>
       <c r="R646" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S646" s="13" t="inlineStr">
@@ -63591,7 +63591,7 @@
       </c>
       <c r="R648" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S648" s="13" t="inlineStr">
@@ -63688,7 +63688,7 @@
       </c>
       <c r="R649" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S649" s="13" t="inlineStr">
@@ -64076,7 +64076,7 @@
       </c>
       <c r="R653" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S653" s="13" t="inlineStr">
@@ -64270,7 +64270,7 @@
       </c>
       <c r="R655" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S655" s="13" t="inlineStr">
@@ -64367,7 +64367,7 @@
       </c>
       <c r="R656" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S656" s="13" t="inlineStr">
@@ -64464,7 +64464,7 @@
       </c>
       <c r="R657" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S657" s="13" t="inlineStr">
@@ -64658,7 +64658,7 @@
       </c>
       <c r="R659" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S659" s="13" t="inlineStr">
@@ -64755,7 +64755,7 @@
       </c>
       <c r="R660" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S660" s="13" t="inlineStr">
@@ -64852,7 +64852,7 @@
       </c>
       <c r="R661" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S661" s="13" t="inlineStr">
@@ -64949,7 +64949,7 @@
       </c>
       <c r="R662" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S662" s="13" t="inlineStr">
@@ -65046,7 +65046,7 @@
       </c>
       <c r="R663" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S663" s="13" t="inlineStr">
@@ -65143,7 +65143,7 @@
       </c>
       <c r="R664" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S664" s="13" t="inlineStr">
@@ -65240,7 +65240,7 @@
       </c>
       <c r="R665" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S665" s="13" t="inlineStr">
@@ -65337,7 +65337,7 @@
       </c>
       <c r="R666" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S666" s="13" t="inlineStr">
@@ -65434,7 +65434,7 @@
       </c>
       <c r="R667" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S667" s="13" t="inlineStr">
@@ -65531,7 +65531,7 @@
       </c>
       <c r="R668" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S668" s="13" t="inlineStr">
@@ -65725,7 +65725,7 @@
       </c>
       <c r="R670" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S670" s="13" t="inlineStr">
@@ -65822,7 +65822,7 @@
       </c>
       <c r="R671" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S671" s="13" t="inlineStr">
@@ -67665,7 +67665,7 @@
       </c>
       <c r="R690" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S690" s="15" t="inlineStr">
@@ -67762,7 +67762,7 @@
       </c>
       <c r="R691" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S691" s="15" t="inlineStr">
@@ -67859,7 +67859,7 @@
       </c>
       <c r="R692" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S692" s="15" t="inlineStr">
@@ -68150,7 +68150,7 @@
       </c>
       <c r="R695" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S695" s="15" t="inlineStr">
@@ -68344,7 +68344,7 @@
       </c>
       <c r="R697" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S697" s="15" t="inlineStr">
@@ -68441,7 +68441,7 @@
       </c>
       <c r="R698" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S698" s="15" t="inlineStr">
@@ -68635,7 +68635,7 @@
       </c>
       <c r="R700" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S700" s="15" t="inlineStr">
@@ -68732,7 +68732,7 @@
       </c>
       <c r="R701" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S701" s="15" t="inlineStr">
@@ -68926,7 +68926,7 @@
       </c>
       <c r="R703" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S703" s="15" t="inlineStr">
@@ -69023,7 +69023,7 @@
       </c>
       <c r="R704" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S704" s="15" t="inlineStr">
@@ -69120,7 +69120,7 @@
       </c>
       <c r="R705" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S705" s="15" t="inlineStr">
@@ -69217,7 +69217,7 @@
       </c>
       <c r="R706" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S706" s="15" t="inlineStr">
@@ -69314,7 +69314,7 @@
       </c>
       <c r="R707" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S707" s="15" t="inlineStr">
@@ -69896,7 +69896,7 @@
       </c>
       <c r="R713" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S713" s="15" t="inlineStr">
@@ -71254,7 +71254,7 @@
       </c>
       <c r="R727" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S727" s="15" t="inlineStr">
@@ -72418,7 +72418,7 @@
       </c>
       <c r="R739" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S739" s="15" t="inlineStr">
@@ -72806,7 +72806,7 @@
       </c>
       <c r="R743" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S743" s="15" t="inlineStr">
@@ -72903,7 +72903,7 @@
       </c>
       <c r="R744" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S744" s="15" t="inlineStr">
@@ -74746,7 +74746,7 @@
       </c>
       <c r="R763" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S763" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Verify 91 more Draft words with sources (batch 2); fix 4 meanings
- 순위발표식: ranking rounds happen throughout a survival show, not only the finale
- 초동: first-week sales (not 'first-day-and-week')
- 자컨: agency-produced in-house content, not idols' self-made clips
- 만능돌: all-rounder incl. variety/acting, not just singing/dancing/rap/visuals
- zh-CN: 重要指针 -> 重要指标 (OpenCC mis-conversion)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$770</definedName>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="R12" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S12" s="7" t="inlineStr">
@@ -2033,27 +2033,27 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Casual behind-the-scenes content idols make and post themselves.</t>
+          <t>Short for 자체 콘텐츠 — videos a group's agency plans and produces in-house, like the group's own variety shows, vlogs and behind-the-scenes clips.</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Contenido casual detrás de cámaras que los ídolos crean y publican ellos mismos.</t>
+          <t>Abreviatura de 자체 콘텐츠: videos que la agencia del grupo planea y produce por su cuenta, como sus propios programas de variedades, vlogs y clips detrás de cámaras.</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>偶像自己拍攝並上傳的輕鬆幕後內容。</t>
+          <t>「自體內容」的縮寫——經紀公司自己企劃、自製的偶像影片，例如團體自製綜藝、vlog和幕後花絮。</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>偶像自己拍摄并上传的轻松幕后内容。</t>
+          <t>“自体内容”的缩写——经纪公司自己企划、自制的偶像视频，例如团体自制综艺、vlog和幕后花絮。</t>
         </is>
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>アイドルが自分で撮影して投稿する気軽な舞台裏コンテンツ。</t>
+          <t>「自体コンテンツ」の略。事務所が自ら企画・制作するアイドルの映像コンテンツで、グループの自主制作バラエティやVlog、舞台裏映像など。</t>
         </is>
       </c>
       <c r="K14" s="8" t="inlineStr">
@@ -2093,7 +2093,7 @@
       </c>
       <c r="R14" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S14" s="7" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="R18" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S18" s="7" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="R19" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S19" s="7" t="inlineStr">
@@ -3548,7 +3548,7 @@
       </c>
       <c r="R29" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S29" s="7" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="R32" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S32" s="7" t="inlineStr">
@@ -3936,7 +3936,7 @@
       </c>
       <c r="R33" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S33" s="7" t="inlineStr">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="R34" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S34" s="7" t="inlineStr">
@@ -4421,7 +4421,7 @@
       </c>
       <c r="R38" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S38" s="7" t="inlineStr">
@@ -5488,7 +5488,7 @@
       </c>
       <c r="R49" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S49" s="7" t="inlineStr">
@@ -5585,7 +5585,7 @@
       </c>
       <c r="R50" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S50" s="7" t="inlineStr">
@@ -6361,7 +6361,7 @@
       </c>
       <c r="R58" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S58" s="7" t="inlineStr">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="R59" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S59" s="7" t="inlineStr">
@@ -7331,7 +7331,7 @@
       </c>
       <c r="R68" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S68" s="7" t="inlineStr">
@@ -7428,7 +7428,7 @@
       </c>
       <c r="R69" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S69" s="7" t="inlineStr">
@@ -7525,7 +7525,7 @@
       </c>
       <c r="R70" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S70" s="7" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </c>
       <c r="R71" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S71" s="7" t="inlineStr">
@@ -8241,27 +8241,27 @@
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
-          <t>An "all-rounder idol" skilled across singing, dancing, rapping, and visuals.</t>
+          <t>An "all-rounder idol" — good at everything: on stage, and also in variety shows, acting and more.</t>
         </is>
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
-          <t>Un "ídolo todoterreno", talentoso en canto, baile, rap y también en apariencia.</t>
+          <t>Un "ídolo todoterreno": bueno en todo, en el escenario y también en programas de variedades, actuación y más.</t>
         </is>
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t>在唱歌、跳舞、饒舌、visual各方面都很全面的「全能偶像」。</t>
+          <t>舞台之外，綜藝、演戲等各方面也都很拿手的「全能偶像」。</t>
         </is>
       </c>
       <c r="I78" s="8" t="inlineStr">
         <is>
-          <t>在唱歌、跳舞、饶舌、visual各方面都很全面的“全能偶像”。</t>
+          <t>舞台之外，综艺、演戏等各方面也都很拿手的“全能偶像”。</t>
         </is>
       </c>
       <c r="J78" s="8" t="inlineStr">
         <is>
-          <t>歌、ダンス、ラップ、ビジュアルすべてに秀でた「万能アイドル」。</t>
+          <t>ステージだけでなく、バラエティや演技などなんでもこなす「万能アイドル」。</t>
         </is>
       </c>
       <c r="K78" s="8" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="R78" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S78" s="7" t="inlineStr">
@@ -9271,7 +9271,7 @@
       </c>
       <c r="R88" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S88" s="7" t="inlineStr">
@@ -9368,7 +9368,7 @@
       </c>
       <c r="R89" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S89" s="7" t="inlineStr">
@@ -10375,12 +10375,12 @@
       </c>
       <c r="F100" s="8" t="inlineStr">
         <is>
-          <t>Short for "first-day-and-week sales" — an album's initial sales figures, a key chart metric.</t>
+          <t>Short for 초동 판매량 (initial sales) — an album's sales in its first week from release, a key chart metric.</t>
         </is>
       </c>
       <c r="G100" s="8" t="inlineStr">
         <is>
-          <t>Abreviatura de "ventas del primer día y semana": las cifras de ventas iniciales de un álbum, una métrica clave de las listas.</t>
+          <t>Abreviatura de 초동 판매량 (ventas iniciales): las ventas de un álbum en su primera semana desde el lanzamiento, una métrica clave de las listas.</t>
         </is>
       </c>
       <c r="H100" s="8" t="inlineStr">
@@ -10390,12 +10390,12 @@
       </c>
       <c r="I100" s="8" t="inlineStr">
         <is>
-          <t>“初动”——专辑发行首周的销量数字，是重要的排行指针。</t>
+          <t>“初动”——专辑发行首周的销量数字，是重要的排行指标。</t>
         </is>
       </c>
       <c r="J100" s="8" t="inlineStr">
         <is>
-          <t>「初日・初週の売り上げ」の略——アルバムの初期販売数を示す、重要なチャート指標。</t>
+          <t>「初動販売量」の略——発売から1週間のアルバム販売枚数のことで、重要なチャート指標。</t>
         </is>
       </c>
       <c r="K100" s="8" t="inlineStr">
@@ -10435,7 +10435,7 @@
       </c>
       <c r="R100" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S100" s="7" t="inlineStr">
@@ -10487,7 +10487,7 @@
       </c>
       <c r="I101" s="8" t="inlineStr">
         <is>
-          <t>美国告示牌音乐排行榜，是K-pop国际成功的重要指针。</t>
+          <t>美国告示牌音乐排行榜，是K-pop国际成功的重要指标。</t>
         </is>
       </c>
       <c r="J101" s="8" t="inlineStr">
@@ -11830,27 +11830,27 @@
       </c>
       <c r="F115" s="8" t="inlineStr">
         <is>
-          <t>The finale round of a survival show where the final debut lineup ranking is revealed live.</t>
+          <t>A ranking announcement round on a survival show, where contestants' current ranks are revealed and those below the cutoff are eliminated.</t>
         </is>
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t>La ronda final de un programa de supervivencia donde se revela en vivo el ranking final de la alineación de debut.</t>
+          <t>La ronda de anuncio de posiciones de un programa de supervivencia, donde se revela el puesto actual de cada concursante y quienes quedan por debajo del corte son eliminados.</t>
         </is>
       </c>
       <c r="H115" s="8" t="inlineStr">
         <is>
-          <t>選秀節目最終回中現場公布最終出道排名的環節。</t>
+          <t>選秀節目中公布參賽者當前排名的環節，排名在淘汰線以下的人會被淘汰。</t>
         </is>
       </c>
       <c r="I115" s="8" t="inlineStr">
         <is>
-          <t>选秀节目最终回中现场公布最终出道排名的环节。</t>
+          <t>选秀节目中公布参赛者当前排名的环节，排名在淘汰线以下的人会被淘汰。</t>
         </is>
       </c>
       <c r="J115" s="8" t="inlineStr">
         <is>
-          <t>サバイバル番組の最終回で、最終的なデビューメンバーの順位がライブで発表される場面。</t>
+          <t>サバイバル番組で参加者の現在の順位が発表され、ボーダー以下の人が脱落する回。</t>
         </is>
       </c>
       <c r="K115" s="8" t="inlineStr">
@@ -11865,7 +11865,7 @@
       </c>
       <c r="M115" s="8" t="inlineStr">
         <is>
-          <t>Todos lloramos juntos viendo la ceremonia de revelación del ranking final.</t>
+          <t>Todos lloramos juntos viendo la ceremonia de anuncio de posiciones.</t>
         </is>
       </c>
       <c r="N115" s="8" t="inlineStr">
@@ -11885,12 +11885,12 @@
       </c>
       <c r="Q115" s="8" t="inlineStr">
         <is>
-          <t>Survival show finales</t>
+          <t>Survival shows</t>
         </is>
       </c>
       <c r="R115" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S115" s="7" t="inlineStr">
@@ -12084,7 +12084,7 @@
       </c>
       <c r="R117" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S117" s="7" t="inlineStr">
@@ -12375,7 +12375,7 @@
       </c>
       <c r="R120" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S120" s="7" t="inlineStr">
@@ -12472,7 +12472,7 @@
       </c>
       <c r="R121" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S121" s="7" t="inlineStr">
@@ -15479,7 +15479,7 @@
       </c>
       <c r="R152" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S152" s="7" t="inlineStr">
@@ -15576,7 +15576,7 @@
       </c>
       <c r="R153" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S153" s="7" t="inlineStr">
@@ -15867,7 +15867,7 @@
       </c>
       <c r="R156" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S156" s="7" t="inlineStr">
@@ -15964,7 +15964,7 @@
       </c>
       <c r="R157" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S157" s="7" t="inlineStr">
@@ -16158,7 +16158,7 @@
       </c>
       <c r="R159" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S159" s="7" t="inlineStr">
@@ -16255,7 +16255,7 @@
       </c>
       <c r="R160" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S160" s="7" t="inlineStr">
@@ -16449,7 +16449,7 @@
       </c>
       <c r="R162" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S162" s="7" t="inlineStr">
@@ -16643,7 +16643,7 @@
       </c>
       <c r="R164" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S164" s="7" t="inlineStr">
@@ -16934,7 +16934,7 @@
       </c>
       <c r="R167" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S167" s="7" t="inlineStr">
@@ -17128,7 +17128,7 @@
       </c>
       <c r="R169" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S169" s="7" t="inlineStr">
@@ -19262,7 +19262,7 @@
       </c>
       <c r="R191" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S191" s="9" t="inlineStr">
@@ -21687,7 +21687,7 @@
       </c>
       <c r="R216" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S216" s="9" t="inlineStr">
@@ -22754,7 +22754,7 @@
       </c>
       <c r="R227" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S227" s="9" t="inlineStr">
@@ -23142,7 +23142,7 @@
       </c>
       <c r="R231" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S231" s="9" t="inlineStr">
@@ -23433,7 +23433,7 @@
       </c>
       <c r="R234" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S234" s="9" t="inlineStr">
@@ -24888,7 +24888,7 @@
       </c>
       <c r="R249" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S249" s="9" t="inlineStr">
@@ -25567,7 +25567,7 @@
       </c>
       <c r="R256" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S256" s="9" t="inlineStr">
@@ -26925,7 +26925,7 @@
       </c>
       <c r="R270" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S270" s="9" t="inlineStr">
@@ -27992,7 +27992,7 @@
       </c>
       <c r="R281" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S281" s="9" t="inlineStr">
@@ -28283,7 +28283,7 @@
       </c>
       <c r="R284" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S284" s="9" t="inlineStr">
@@ -29156,7 +29156,7 @@
       </c>
       <c r="R293" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S293" s="9" t="inlineStr">
@@ -29544,7 +29544,7 @@
       </c>
       <c r="R297" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S297" s="9" t="inlineStr">
@@ -29641,7 +29641,7 @@
       </c>
       <c r="R298" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S298" s="9" t="inlineStr">
@@ -29932,7 +29932,7 @@
       </c>
       <c r="R301" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S301" s="9" t="inlineStr">
@@ -30126,7 +30126,7 @@
       </c>
       <c r="R303" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S303" s="9" t="inlineStr">
@@ -30417,7 +30417,7 @@
       </c>
       <c r="R306" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S306" s="9" t="inlineStr">
@@ -35073,7 +35073,7 @@
       </c>
       <c r="R354" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S354" s="11" t="inlineStr">
@@ -35170,7 +35170,7 @@
       </c>
       <c r="R355" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S355" s="11" t="inlineStr">
@@ -35849,7 +35849,7 @@
       </c>
       <c r="R362" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S362" s="11" t="inlineStr">
@@ -36043,7 +36043,7 @@
       </c>
       <c r="R364" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S364" s="11" t="inlineStr">
@@ -36140,7 +36140,7 @@
       </c>
       <c r="R365" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S365" s="11" t="inlineStr">
@@ -36237,7 +36237,7 @@
       </c>
       <c r="R366" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S366" s="11" t="inlineStr">
@@ -36334,7 +36334,7 @@
       </c>
       <c r="R367" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S367" s="11" t="inlineStr">
@@ -36722,7 +36722,7 @@
       </c>
       <c r="R371" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S371" s="11" t="inlineStr">
@@ -36819,7 +36819,7 @@
       </c>
       <c r="R372" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S372" s="11" t="inlineStr">
@@ -36916,7 +36916,7 @@
       </c>
       <c r="R373" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S373" s="11" t="inlineStr">
@@ -37013,7 +37013,7 @@
       </c>
       <c r="R374" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S374" s="11" t="inlineStr">
@@ -37110,7 +37110,7 @@
       </c>
       <c r="R375" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S375" s="11" t="inlineStr">
@@ -37207,7 +37207,7 @@
       </c>
       <c r="R376" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S376" s="11" t="inlineStr">
@@ -37401,7 +37401,7 @@
       </c>
       <c r="R378" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S378" s="11" t="inlineStr">
@@ -37498,7 +37498,7 @@
       </c>
       <c r="R379" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S379" s="11" t="inlineStr">
@@ -37595,7 +37595,7 @@
       </c>
       <c r="R380" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S380" s="11" t="inlineStr">
@@ -38080,7 +38080,7 @@
       </c>
       <c r="R385" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S385" s="11" t="inlineStr">
@@ -38177,7 +38177,7 @@
       </c>
       <c r="R386" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S386" s="11" t="inlineStr">
@@ -39341,7 +39341,7 @@
       </c>
       <c r="R398" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S398" s="11" t="inlineStr">
@@ -39438,7 +39438,7 @@
       </c>
       <c r="R399" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S399" s="11" t="inlineStr">
@@ -39535,7 +39535,7 @@
       </c>
       <c r="R400" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S400" s="11" t="inlineStr">
@@ -39632,7 +39632,7 @@
       </c>
       <c r="R401" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S401" s="11" t="inlineStr">
@@ -39826,7 +39826,7 @@
       </c>
       <c r="R403" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S403" s="11" t="inlineStr">
@@ -39923,7 +39923,7 @@
       </c>
       <c r="R404" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S404" s="11" t="inlineStr">
@@ -40117,7 +40117,7 @@
       </c>
       <c r="R406" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S406" s="11" t="inlineStr">
@@ -40505,7 +40505,7 @@
       </c>
       <c r="R410" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S410" s="11" t="inlineStr">
@@ -40893,7 +40893,7 @@
       </c>
       <c r="R414" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S414" s="11" t="inlineStr">
@@ -41184,7 +41184,7 @@
       </c>
       <c r="R417" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S417" s="11" t="inlineStr">
@@ -67374,7 +67374,7 @@
       </c>
       <c r="R687" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S687" s="15" t="inlineStr">
@@ -67471,7 +67471,7 @@
       </c>
       <c r="R688" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S688" s="15" t="inlineStr">
@@ -67956,7 +67956,7 @@
       </c>
       <c r="R693" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S693" s="15" t="inlineStr">
@@ -68247,7 +68247,7 @@
       </c>
       <c r="R696" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S696" s="15" t="inlineStr">
@@ -68538,7 +68538,7 @@
       </c>
       <c r="R699" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S699" s="15" t="inlineStr">
@@ -69508,7 +69508,7 @@
       </c>
       <c r="R709" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S709" s="15" t="inlineStr">
@@ -69702,7 +69702,7 @@
       </c>
       <c r="R711" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S711" s="15" t="inlineStr">
@@ -70187,7 +70187,7 @@
       </c>
       <c r="R716" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S716" s="15" t="inlineStr">
@@ -71739,7 +71739,7 @@
       </c>
       <c r="R732" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S732" s="15" t="inlineStr">
@@ -71933,7 +71933,7 @@
       </c>
       <c r="R734" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S734" s="15" t="inlineStr">
@@ -72515,7 +72515,7 @@
       </c>
       <c r="R740" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S740" s="15" t="inlineStr">
@@ -74649,7 +74649,7 @@
       </c>
       <c r="R762" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S762" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Verify 20 more Draft words with sources (batch 3)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$770</definedName>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="R17" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S17" s="7" t="inlineStr">
@@ -5003,7 +5003,7 @@
       </c>
       <c r="R44" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S44" s="7" t="inlineStr">
@@ -5294,7 +5294,7 @@
       </c>
       <c r="R47" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S47" s="7" t="inlineStr">
@@ -10047,7 +10047,7 @@
       </c>
       <c r="R96" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S96" s="7" t="inlineStr">
@@ -10629,7 +10629,7 @@
       </c>
       <c r="R102" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S102" s="7" t="inlineStr">
@@ -10726,7 +10726,7 @@
       </c>
       <c r="R103" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S103" s="7" t="inlineStr">
@@ -10823,7 +10823,7 @@
       </c>
       <c r="R104" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S104" s="7" t="inlineStr">
@@ -11211,7 +11211,7 @@
       </c>
       <c r="R108" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S108" s="7" t="inlineStr">
@@ -12569,7 +12569,7 @@
       </c>
       <c r="R122" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S122" s="7" t="inlineStr">
@@ -12666,7 +12666,7 @@
       </c>
       <c r="R123" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S123" s="7" t="inlineStr">
@@ -12957,7 +12957,7 @@
       </c>
       <c r="R126" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S126" s="7" t="inlineStr">
@@ -13054,7 +13054,7 @@
       </c>
       <c r="R127" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S127" s="7" t="inlineStr">
@@ -13151,7 +13151,7 @@
       </c>
       <c r="R128" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S128" s="7" t="inlineStr">
@@ -13248,7 +13248,7 @@
       </c>
       <c r="R129" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S129" s="7" t="inlineStr">
@@ -14121,7 +14121,7 @@
       </c>
       <c r="R138" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S138" s="7" t="inlineStr">
@@ -16837,7 +16837,7 @@
       </c>
       <c r="R166" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S166" s="7" t="inlineStr">
@@ -17322,7 +17322,7 @@
       </c>
       <c r="R171" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S171" s="7" t="inlineStr">
@@ -43706,7 +43706,7 @@
       </c>
       <c r="R443" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S443" s="13" t="inlineStr">
@@ -66501,7 +66501,7 @@
       </c>
       <c r="R678" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S678" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Verify 55 more draft words with sources; fix 안습 meaning in all languages
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$770</definedName>
@@ -5391,7 +5391,7 @@
       </c>
       <c r="R48" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S48" s="7" t="inlineStr">
@@ -5876,7 +5876,7 @@
       </c>
       <c r="R53" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S53" s="7" t="inlineStr">
@@ -8010,7 +8010,7 @@
       </c>
       <c r="R75" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S75" s="7" t="inlineStr">
@@ -8107,7 +8107,7 @@
       </c>
       <c r="R76" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S76" s="7" t="inlineStr">
@@ -8398,7 +8398,7 @@
       </c>
       <c r="R79" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S79" s="7" t="inlineStr">
@@ -8495,7 +8495,7 @@
       </c>
       <c r="R80" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S80" s="7" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="R81" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S81" s="7" t="inlineStr">
@@ -8786,7 +8786,7 @@
       </c>
       <c r="R83" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S83" s="7" t="inlineStr">
@@ -8883,7 +8883,7 @@
       </c>
       <c r="R84" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S84" s="7" t="inlineStr">
@@ -8980,7 +8980,7 @@
       </c>
       <c r="R85" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S85" s="7" t="inlineStr">
@@ -9465,7 +9465,7 @@
       </c>
       <c r="R90" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S90" s="7" t="inlineStr">
@@ -9562,7 +9562,7 @@
       </c>
       <c r="R91" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S91" s="7" t="inlineStr">
@@ -11308,7 +11308,7 @@
       </c>
       <c r="R109" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S109" s="7" t="inlineStr">
@@ -11696,7 +11696,7 @@
       </c>
       <c r="R113" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S113" s="7" t="inlineStr">
@@ -12763,7 +12763,7 @@
       </c>
       <c r="R124" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S124" s="7" t="inlineStr">
@@ -13733,7 +13733,7 @@
       </c>
       <c r="R134" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S134" s="7" t="inlineStr">
@@ -14994,7 +14994,7 @@
       </c>
       <c r="R147" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S147" s="7" t="inlineStr">
@@ -15770,7 +15770,7 @@
       </c>
       <c r="R155" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S155" s="7" t="inlineStr">
@@ -19650,7 +19650,7 @@
       </c>
       <c r="R195" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S195" s="9" t="inlineStr">
@@ -19747,7 +19747,7 @@
       </c>
       <c r="R196" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S196" s="9" t="inlineStr">
@@ -19844,7 +19844,7 @@
       </c>
       <c r="R197" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S197" s="9" t="inlineStr">
@@ -22851,7 +22851,7 @@
       </c>
       <c r="R228" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S228" s="9" t="inlineStr">
@@ -23336,7 +23336,7 @@
       </c>
       <c r="R233" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S233" s="9" t="inlineStr">
@@ -26149,7 +26149,7 @@
       </c>
       <c r="R262" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S262" s="9" t="inlineStr">
@@ -29447,7 +29447,7 @@
       </c>
       <c r="R296" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S296" s="9" t="inlineStr">
@@ -29835,7 +29835,7 @@
       </c>
       <c r="R300" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S300" s="9" t="inlineStr">
@@ -30999,7 +30999,7 @@
       </c>
       <c r="R312" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S312" s="11" t="inlineStr">
@@ -31036,27 +31036,27 @@
       </c>
       <c r="F313" s="12" t="inlineStr">
         <is>
-          <t>Literally "eyes moist" — describes something pitiful or embarrassing.</t>
+          <t>Short for 안구에 습기 ("moisture in the eyes") — something so sad or pitiful it almost brings tears; often used half-jokingly.</t>
         </is>
       </c>
       <c r="G313" s="12" t="inlineStr">
         <is>
-          <t>Literalmente "ojos húmedos", describe algo lamentable o vergonzoso.</t>
+          <t>Abreviatura de 안구에 습기 ("humedad en los ojos"): algo tan triste o lamentable que casi hace llorar; a menudo se dice medio en broma.</t>
         </is>
       </c>
       <c r="H313" s="12" t="inlineStr">
         <is>
-          <t>字面意思是「眼睛濕了」——形容可憐或尷尬的事，淚目。</t>
+          <t>「안구에 습기」（眼球有濕氣）的縮寫——形容可憐、悲傷到快要流淚的事，常帶點半開玩笑的語氣。</t>
         </is>
       </c>
       <c r="I313" s="12" t="inlineStr">
         <is>
-          <t>字面意思是“眼睛湿了”——形容可怜或尴尬的事，泪目。</t>
+          <t>“안구에 습기”（眼球有湿气）的缩写——形容可怜、悲伤到快要流泪的事，常带点半开玩笑的语气。</t>
         </is>
       </c>
       <c r="J313" s="12" t="inlineStr">
         <is>
-          <t>直訳すると「目が濡れる」——哀れ、または恥ずかしいことを表す。</t>
+          <t>「안구에 습기（眼球に湿気）」の略——涙が出そうなほど哀れ・悲しいことを表す。半分冗談っぽく使うことが多い。</t>
         </is>
       </c>
       <c r="K313" s="12" t="inlineStr">
@@ -31096,7 +31096,7 @@
       </c>
       <c r="R313" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S313" s="11" t="inlineStr">
@@ -31193,7 +31193,7 @@
       </c>
       <c r="R314" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S314" s="11" t="inlineStr">
@@ -31290,7 +31290,7 @@
       </c>
       <c r="R315" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S315" s="11" t="inlineStr">
@@ -31484,7 +31484,7 @@
       </c>
       <c r="R317" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S317" s="11" t="inlineStr">
@@ -32745,7 +32745,7 @@
       </c>
       <c r="R330" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S330" s="11" t="inlineStr">
@@ -33521,7 +33521,7 @@
       </c>
       <c r="R338" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S338" s="11" t="inlineStr">
@@ -33618,7 +33618,7 @@
       </c>
       <c r="R339" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S339" s="11" t="inlineStr">
@@ -34006,7 +34006,7 @@
       </c>
       <c r="R343" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S343" s="11" t="inlineStr">
@@ -34685,7 +34685,7 @@
       </c>
       <c r="R350" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S350" s="11" t="inlineStr">
@@ -34976,7 +34976,7 @@
       </c>
       <c r="R353" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S353" s="11" t="inlineStr">
@@ -35752,7 +35752,7 @@
       </c>
       <c r="R361" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S361" s="11" t="inlineStr">
@@ -36625,7 +36625,7 @@
       </c>
       <c r="R370" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S370" s="11" t="inlineStr">
@@ -38468,7 +38468,7 @@
       </c>
       <c r="R389" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S389" s="11" t="inlineStr">
@@ -40602,7 +40602,7 @@
       </c>
       <c r="R411" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S411" s="11" t="inlineStr">
@@ -41281,7 +41281,7 @@
       </c>
       <c r="R418" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S418" s="11" t="inlineStr">
@@ -41766,7 +41766,7 @@
       </c>
       <c r="R423" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S423" s="11" t="inlineStr">
@@ -42154,7 +42154,7 @@
       </c>
       <c r="R427" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S427" s="11" t="inlineStr">
@@ -42348,7 +42348,7 @@
       </c>
       <c r="R429" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S429" s="11" t="inlineStr">
@@ -69411,7 +69411,7 @@
       </c>
       <c r="R708" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S708" s="15" t="inlineStr">
@@ -69605,7 +69605,7 @@
       </c>
       <c r="R710" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S710" s="15" t="inlineStr">
@@ -70284,7 +70284,7 @@
       </c>
       <c r="R717" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S717" s="15" t="inlineStr">
@@ -70575,7 +70575,7 @@
       </c>
       <c r="R720" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S720" s="15" t="inlineStr">
@@ -70769,7 +70769,7 @@
       </c>
       <c r="R722" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S722" s="15" t="inlineStr">
@@ -71448,7 +71448,7 @@
       </c>
       <c r="R729" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S729" s="15" t="inlineStr">
@@ -71642,7 +71642,7 @@
       </c>
       <c r="R731" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S731" s="15" t="inlineStr">
@@ -72030,7 +72030,7 @@
       </c>
       <c r="R735" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S735" s="15" t="inlineStr">
@@ -74552,7 +74552,7 @@
       </c>
       <c r="R761" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S761" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Verify 41 more draft words with sources; fix 남친룩 meaning in all languages
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$770</definedName>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="R25" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S25" s="7" t="inlineStr">
@@ -3742,7 +3742,7 @@
       </c>
       <c r="R31" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S31" s="7" t="inlineStr">
@@ -5100,7 +5100,7 @@
       </c>
       <c r="R45" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S45" s="7" t="inlineStr">
@@ -5973,7 +5973,7 @@
       </c>
       <c r="R54" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S54" s="7" t="inlineStr">
@@ -6070,7 +6070,7 @@
       </c>
       <c r="R55" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S55" s="7" t="inlineStr">
@@ -6167,7 +6167,7 @@
       </c>
       <c r="R56" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S56" s="7" t="inlineStr">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="R57" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S57" s="7" t="inlineStr">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="R61" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S61" s="7" t="inlineStr">
@@ -7137,7 +7137,7 @@
       </c>
       <c r="R66" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S66" s="7" t="inlineStr">
@@ -7913,7 +7913,7 @@
       </c>
       <c r="R74" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S74" s="7" t="inlineStr">
@@ -10338,7 +10338,7 @@
       </c>
       <c r="R99" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S99" s="7" t="inlineStr">
@@ -10532,7 +10532,7 @@
       </c>
       <c r="R101" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S101" s="7" t="inlineStr">
@@ -10920,7 +10920,7 @@
       </c>
       <c r="R105" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S105" s="7" t="inlineStr">
@@ -11114,7 +11114,7 @@
       </c>
       <c r="R107" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S107" s="7" t="inlineStr">
@@ -14024,7 +14024,7 @@
       </c>
       <c r="R137" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S137" s="7" t="inlineStr">
@@ -14412,7 +14412,7 @@
       </c>
       <c r="R141" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S141" s="7" t="inlineStr">
@@ -14509,7 +14509,7 @@
       </c>
       <c r="R142" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S142" s="7" t="inlineStr">
@@ -15188,7 +15188,7 @@
       </c>
       <c r="R149" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S149" s="7" t="inlineStr">
@@ -16061,7 +16061,7 @@
       </c>
       <c r="R158" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S158" s="7" t="inlineStr">
@@ -16546,7 +16546,7 @@
       </c>
       <c r="R163" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S163" s="7" t="inlineStr">
@@ -18971,7 +18971,7 @@
       </c>
       <c r="R188" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S188" s="9" t="inlineStr">
@@ -23530,7 +23530,7 @@
       </c>
       <c r="R235" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S235" s="9" t="inlineStr">
@@ -24500,7 +24500,7 @@
       </c>
       <c r="R245" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S245" s="9" t="inlineStr">
@@ -26537,7 +26537,7 @@
       </c>
       <c r="R266" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S266" s="9" t="inlineStr">
@@ -32454,7 +32454,7 @@
       </c>
       <c r="R327" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S327" s="11" t="inlineStr">
@@ -35461,7 +35461,7 @@
       </c>
       <c r="R358" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S358" s="11" t="inlineStr">
@@ -36431,7 +36431,7 @@
       </c>
       <c r="R368" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S368" s="11" t="inlineStr">
@@ -36528,7 +36528,7 @@
       </c>
       <c r="R369" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S369" s="11" t="inlineStr">
@@ -40990,7 +40990,7 @@
       </c>
       <c r="R415" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S415" s="11" t="inlineStr">
@@ -41378,7 +41378,7 @@
       </c>
       <c r="R419" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S419" s="11" t="inlineStr">
@@ -42057,7 +42057,7 @@
       </c>
       <c r="R426" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S426" s="11" t="inlineStr">
@@ -49623,7 +49623,7 @@
       </c>
       <c r="R504" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S504" s="13" t="inlineStr">
@@ -52824,7 +52824,7 @@
       </c>
       <c r="R537" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S537" s="13" t="inlineStr">
@@ -53115,7 +53115,7 @@
       </c>
       <c r="R540" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S540" s="13" t="inlineStr">
@@ -60972,7 +60972,7 @@
       </c>
       <c r="R621" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S621" s="13" t="inlineStr">
@@ -63494,7 +63494,7 @@
       </c>
       <c r="R647" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S647" s="13" t="inlineStr">
@@ -70478,7 +70478,7 @@
       </c>
       <c r="R719" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S719" s="15" t="inlineStr">
@@ -71157,7 +71157,7 @@
       </c>
       <c r="R726" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S726" s="15" t="inlineStr">
@@ -73000,7 +73000,7 @@
       </c>
       <c r="R745" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S745" s="15" t="inlineStr">
@@ -73037,57 +73037,57 @@
       </c>
       <c r="F746" s="16" t="inlineStr">
         <is>
-          <t>"Boyfriend look" — a fashion style mimicking oversized, borrowed-looking boyfriend clothing.</t>
+          <t>"Boyfriend look" — a guy's outfit or vibe that makes him look like the ideal boyfriend on a date; fans also use it for idol photos that feel like a date.</t>
         </is>
       </c>
       <c r="G746" s="16" t="inlineStr">
         <is>
-          <t>"Look de novio": un estilo de moda que imita ropa holgada, como si fuera prestada por el novio.</t>
+          <t>"Look de novio": el outfit o la vibra de un chico que lo hace ver como el novio ideal en una cita; los fans también lo usan para fotos de idols que parecen de una cita.</t>
         </is>
       </c>
       <c r="H746" s="16" t="inlineStr">
         <is>
-          <t>「男友風」——模仿男友寬鬆、彷彿借穿男友衣服的穿搭風格。</t>
+          <t>「男友風」——男生看起來像約會中理想男友的穿搭或氛圍；粉絲也用來形容像約會照的偶像照片。</t>
         </is>
       </c>
       <c r="I746" s="16" t="inlineStr">
         <is>
-          <t>“男友风”——模仿男友宽松、仿佛借穿男友衣服的穿搭风格。</t>
+          <t>“男友风”——男生看起来像约会中理想男友的穿搭或氛围；粉丝也用来形容像约会照的偶像照片。</t>
         </is>
       </c>
       <c r="J746" s="16" t="inlineStr">
         <is>
-          <t>「彼氏ルック」——彼氏の服を借りたような、オーバーサイズのファッションスタイル。</t>
+          <t>「彼氏ルック」——デート中の理想の彼氏みたいに見える男性の服装や雰囲気。デートっぽいアイドルの写真にも使う。</t>
         </is>
       </c>
       <c r="K746" s="16" t="inlineStr">
         <is>
-          <t>오늘 남친룩으로 입어봤어.</t>
+          <t>이 사진 완전 남친룩이다.</t>
         </is>
       </c>
       <c r="L746" s="16" t="inlineStr">
         <is>
-          <t>I tried out the boyfriend-look style today.</t>
+          <t>This photo is total boyfriend look.</t>
         </is>
       </c>
       <c r="M746" s="16" t="inlineStr">
         <is>
-          <t>Hoy probé el estilo de ropa prestada del novio.</t>
+          <t>Esta foto es puro look de novio.</t>
         </is>
       </c>
       <c r="N746" s="16" t="inlineStr">
         <is>
-          <t>今天試了男友風穿搭。</t>
+          <t>這張照片完全是男友風。</t>
         </is>
       </c>
       <c r="O746" s="16" t="inlineStr">
         <is>
-          <t>今天试了男友风穿搭。</t>
+          <t>这张照片完全是男友风。</t>
         </is>
       </c>
       <c r="P746" s="16" t="inlineStr">
         <is>
-          <t>今日、彼シャツ風の格好してみた。</t>
+          <t>この写真、完全に彼氏ルックだ。</t>
         </is>
       </c>
       <c r="Q746" s="16" t="inlineStr">
@@ -73097,7 +73097,7 @@
       </c>
       <c r="R746" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S746" s="15" t="inlineStr">
@@ -73388,7 +73388,7 @@
       </c>
       <c r="R749" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S749" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Verify 46 more draft words with sources; fix 커플템 meaning in all languages
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$770</definedName>
@@ -5197,7 +5197,7 @@
       </c>
       <c r="R46" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S46" s="7" t="inlineStr">
@@ -13442,7 +13442,7 @@
       </c>
       <c r="R131" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S131" s="7" t="inlineStr">
@@ -14800,7 +14800,7 @@
       </c>
       <c r="R145" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S145" s="7" t="inlineStr">
@@ -19105,57 +19105,57 @@
       </c>
       <c r="F190" s="10" t="inlineStr">
         <is>
-          <t>A "couple item" — matching merch that fans buy to feel paired with their bias or each other.</t>
+          <t>A "couple item" — matching things a couple wears or uses together, like rings, sneakers or phone cases. Fans also joke about having a "couple item" with their bias.</t>
         </is>
       </c>
       <c r="G190" s="10" t="inlineStr">
         <is>
-          <t>Un "artículo de pareja": mercancía a juego que los fans compran para sentirse conectados con su bias u otros fans.</t>
+          <t>Un "artículo de pareja": cosas a juego que una pareja usa junta, como anillos, tenis o fundas de celular. Los fans también bromean con tener un "artículo de pareja" con su bias.</t>
         </is>
       </c>
       <c r="H190" s="10" t="inlineStr">
         <is>
-          <t>「情侶物品」——粉絲購買來與本命或彼此配對的周邊商品。</t>
+          <t>「情侶物品」——情侶一起穿戴或使用的同款物品，像戒指、球鞋、手機殼。粉絲也會開玩笑說和本命用同款是「情侶款」。</t>
         </is>
       </c>
       <c r="I190" s="10" t="inlineStr">
         <is>
-          <t>“情侣物品”——粉丝购买来与本命或彼此配对的周边商品。</t>
+          <t>“情侣物品”——情侣一起穿戴或使用的同款物品，像戒指、球鞋、手机壳。粉丝也会开玩笑说和本命用同款是“情侣款”。</t>
         </is>
       </c>
       <c r="J190" s="10" t="inlineStr">
         <is>
-          <t>推しや互いとペアになった気分を味わうためにファンが買う「カップルアイテム」。</t>
+          <t>「カップルアイテム」——恋人同士でおそろいにする指輪やスニーカー、スマホケースなど。推しと同じ物を持つことを冗談でこう呼ぶファンも。</t>
         </is>
       </c>
       <c r="K190" s="10" t="inlineStr">
         <is>
-          <t>최애랑 커플템 맞춰봤어.</t>
+          <t>남친이랑 커플템 맞췄어.</t>
         </is>
       </c>
       <c r="L190" s="10" t="inlineStr">
         <is>
-          <t>I got a matching couple item with my bias.</t>
+          <t>My boyfriend and I got matching couple items.</t>
         </is>
       </c>
       <c r="M190" s="10" t="inlineStr">
         <is>
-          <t>Conseguí un artículo a juego con mi bias.</t>
+          <t>Mi novio y yo compramos artículos de pareja a juego.</t>
         </is>
       </c>
       <c r="N190" s="10" t="inlineStr">
         <is>
-          <t>跟本命買了情侶小物。</t>
+          <t>跟男朋友買了情侶小物。</t>
         </is>
       </c>
       <c r="O190" s="10" t="inlineStr">
         <is>
-          <t>跟本命买了情侣小物。</t>
+          <t>跟男朋友买了情侣小物。</t>
         </is>
       </c>
       <c r="P190" s="10" t="inlineStr">
         <is>
-          <t>推しとお揃いアイテム合わせてみた。</t>
+          <t>彼氏とペアアイテムそろえた。</t>
         </is>
       </c>
       <c r="Q190" s="10" t="inlineStr">
@@ -19165,7 +19165,7 @@
       </c>
       <c r="R190" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S190" s="9" t="inlineStr">
@@ -22560,7 +22560,7 @@
       </c>
       <c r="R225" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S225" s="9" t="inlineStr">
@@ -22657,7 +22657,7 @@
       </c>
       <c r="R226" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S226" s="9" t="inlineStr">
@@ -23045,7 +23045,7 @@
       </c>
       <c r="R230" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S230" s="9" t="inlineStr">
@@ -23239,7 +23239,7 @@
       </c>
       <c r="R232" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S232" s="9" t="inlineStr">
@@ -23627,7 +23627,7 @@
       </c>
       <c r="R236" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S236" s="9" t="inlineStr">
@@ -23724,7 +23724,7 @@
       </c>
       <c r="R237" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S237" s="9" t="inlineStr">
@@ -24306,7 +24306,7 @@
       </c>
       <c r="R243" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S243" s="9" t="inlineStr">
@@ -25082,7 +25082,7 @@
       </c>
       <c r="R251" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S251" s="9" t="inlineStr">
@@ -25276,7 +25276,7 @@
       </c>
       <c r="R253" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S253" s="9" t="inlineStr">
@@ -25470,7 +25470,7 @@
       </c>
       <c r="R255" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S255" s="9" t="inlineStr">
@@ -25761,7 +25761,7 @@
       </c>
       <c r="R258" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S258" s="9" t="inlineStr">
@@ -28962,7 +28962,7 @@
       </c>
       <c r="R291" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S291" s="9" t="inlineStr">
@@ -34588,7 +34588,7 @@
       </c>
       <c r="R349" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S349" s="11" t="inlineStr">
@@ -34879,7 +34879,7 @@
       </c>
       <c r="R352" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S352" s="11" t="inlineStr">
@@ -38274,7 +38274,7 @@
       </c>
       <c r="R387" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S387" s="11" t="inlineStr">
@@ -38565,7 +38565,7 @@
       </c>
       <c r="R390" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S390" s="11" t="inlineStr">
@@ -39729,7 +39729,7 @@
       </c>
       <c r="R402" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S402" s="11" t="inlineStr">
@@ -40796,7 +40796,7 @@
       </c>
       <c r="R413" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S413" s="11" t="inlineStr">
@@ -41475,7 +41475,7 @@
       </c>
       <c r="R420" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S420" s="11" t="inlineStr">
@@ -41863,7 +41863,7 @@
       </c>
       <c r="R424" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S424" s="11" t="inlineStr">
@@ -51175,7 +51175,7 @@
       </c>
       <c r="R520" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S520" s="13" t="inlineStr">
@@ -61554,7 +61554,7 @@
       </c>
       <c r="R627" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S627" s="13" t="inlineStr">
@@ -63300,7 +63300,7 @@
       </c>
       <c r="R645" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S645" s="13" t="inlineStr">
@@ -67568,7 +67568,7 @@
       </c>
       <c r="R689" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S689" s="15" t="inlineStr">
@@ -68053,7 +68053,7 @@
       </c>
       <c r="R694" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S694" s="15" t="inlineStr">
@@ -68829,7 +68829,7 @@
       </c>
       <c r="R702" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S702" s="15" t="inlineStr">
@@ -69799,7 +69799,7 @@
       </c>
       <c r="R712" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S712" s="15" t="inlineStr">
@@ -69993,7 +69993,7 @@
       </c>
       <c r="R714" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S714" s="15" t="inlineStr">
@@ -70090,7 +70090,7 @@
       </c>
       <c r="R715" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S715" s="15" t="inlineStr">
@@ -70381,7 +70381,7 @@
       </c>
       <c r="R718" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S718" s="15" t="inlineStr">
@@ -70672,7 +70672,7 @@
       </c>
       <c r="R721" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S721" s="15" t="inlineStr">
@@ -71351,7 +71351,7 @@
       </c>
       <c r="R728" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S728" s="15" t="inlineStr">
@@ -72127,7 +72127,7 @@
       </c>
       <c r="R736" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S736" s="15" t="inlineStr">
@@ -72224,7 +72224,7 @@
       </c>
       <c r="R737" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S737" s="15" t="inlineStr">
@@ -73291,7 +73291,7 @@
       </c>
       <c r="R748" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S748" s="15" t="inlineStr">
@@ -73485,7 +73485,7 @@
       </c>
       <c r="R750" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S750" s="15" t="inlineStr">
@@ -73582,7 +73582,7 @@
       </c>
       <c r="R751" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S751" s="15" t="inlineStr">
@@ -73776,7 +73776,7 @@
       </c>
       <c r="R753" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S753" s="15" t="inlineStr">
@@ -73873,7 +73873,7 @@
       </c>
       <c r="R754" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S754" s="15" t="inlineStr">
@@ -74164,7 +74164,7 @@
       </c>
       <c r="R757" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S757" s="15" t="inlineStr">
@@ -74358,7 +74358,7 @@
       </c>
       <c r="R759" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S759" s="15" t="inlineStr">
@@ -74455,7 +74455,7 @@
       </c>
       <c r="R760" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S760" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Verify 41 more draft words with sources; fix 첫콘 meaning in all languages
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$770</definedName>
@@ -4906,7 +4906,7 @@
       </c>
       <c r="R43" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S43" s="7" t="inlineStr">
@@ -5779,7 +5779,7 @@
       </c>
       <c r="R52" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S52" s="7" t="inlineStr">
@@ -7816,7 +7816,7 @@
       </c>
       <c r="R73" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S73" s="7" t="inlineStr">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="R87" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S87" s="7" t="inlineStr">
@@ -11987,7 +11987,7 @@
       </c>
       <c r="R116" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S116" s="7" t="inlineStr">
@@ -12181,7 +12181,7 @@
       </c>
       <c r="R118" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S118" s="7" t="inlineStr">
@@ -12278,7 +12278,7 @@
       </c>
       <c r="R119" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S119" s="7" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="R125" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S125" s="7" t="inlineStr">
@@ -13345,7 +13345,7 @@
       </c>
       <c r="R130" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S130" s="7" t="inlineStr">
@@ -14703,7 +14703,7 @@
       </c>
       <c r="R144" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S144" s="7" t="inlineStr">
@@ -18874,7 +18874,7 @@
       </c>
       <c r="R187" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S187" s="9" t="inlineStr">
@@ -19941,7 +19941,7 @@
       </c>
       <c r="R198" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S198" s="9" t="inlineStr">
@@ -22463,7 +22463,7 @@
       </c>
       <c r="R224" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S224" s="9" t="inlineStr">
@@ -28126,57 +28126,57 @@
       </c>
       <c r="F283" s="10" t="inlineStr">
         <is>
-          <t>Someone's very first time attending a concert for a particular artist — a memorable fan milestone.</t>
+          <t>Short for 첫 콘서트 — the first day of a concert run (the opposite of 막콘). Fans also use it for their own very first concert of an artist.</t>
         </is>
       </c>
       <c r="G283" s="10" t="inlineStr">
         <is>
-          <t>La primera vez que alguien asiste a un concierto de un artista en particular; un hito memorable para un fan.</t>
+          <t>Abreviatura de 첫 콘서트: el primer día de una serie de conciertos (lo contrario de 막콘). Los fans también lo usan para su primer concierto de un artista.</t>
         </is>
       </c>
       <c r="H283" s="10" t="inlineStr">
         <is>
-          <t>某人第一次到現場觀看特定藝人的演唱會，是難忘的追星里程碑。</t>
+          <t>「첫 콘서트」的縮寫——一輪演唱會的首場（相對於막콘）。粉絲也用來指自己第一次去看某藝人的演唱會。</t>
         </is>
       </c>
       <c r="I283" s="10" t="inlineStr">
         <is>
-          <t>某人第一次到现场观看特定艺人的演唱会，是难忘的追星里程碑。</t>
+          <t>“첫 콘서트”的缩写——一轮演唱会的首场（相对于막콘）。粉丝也用来指自己第一次去看某艺人的演唱会。</t>
         </is>
       </c>
       <c r="J283" s="10" t="inlineStr">
         <is>
-          <t>特定のアーティストのコンサートに初めて行くこと——忘れられないファンの節目。</t>
+          <t>첫 콘서트の略——公演期間の初日（막콘の反対）。自分が初めて行くそのアーティストのコンサートの意味でも使う。</t>
         </is>
       </c>
       <c r="K283" s="10" t="inlineStr">
         <is>
-          <t>드디어 첫콘 다녀왔어!</t>
+          <t>첫콘이라 셋리스트 스포 없이 갔어.</t>
         </is>
       </c>
       <c r="L283" s="10" t="inlineStr">
         <is>
-          <t>I finally went to my first concert!</t>
+          <t>It was opening night, so I went in without setlist spoilers.</t>
         </is>
       </c>
       <c r="M283" s="10" t="inlineStr">
         <is>
-          <t>¡Por fin fui a mi primer concierto!</t>
+          <t>Era la primera función, así que fui sin spoilers del setlist.</t>
         </is>
       </c>
       <c r="N283" s="10" t="inlineStr">
         <is>
-          <t>終於去了初次演唱會！</t>
+          <t>因為是首場，沒被歌單劇透就去了。</t>
         </is>
       </c>
       <c r="O283" s="10" t="inlineStr">
         <is>
-          <t>终于去了初次演唱会！</t>
+          <t>因为是首场，没被歌单剧透就去了。</t>
         </is>
       </c>
       <c r="P283" s="10" t="inlineStr">
         <is>
-          <t>ついに初コン行ってきた！</t>
+          <t>初日だからセトリのネタバレなしで行った。</t>
         </is>
       </c>
       <c r="Q283" s="10" t="inlineStr">
@@ -28186,7 +28186,7 @@
       </c>
       <c r="R283" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S283" s="9" t="inlineStr">
@@ -30320,7 +30320,7 @@
       </c>
       <c r="R305" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S305" s="9" t="inlineStr">
@@ -32939,7 +32939,7 @@
       </c>
       <c r="R332" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S332" s="11" t="inlineStr">
@@ -33909,7 +33909,7 @@
       </c>
       <c r="R342" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S342" s="11" t="inlineStr">
@@ -34782,7 +34782,7 @@
       </c>
       <c r="R351" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S351" s="11" t="inlineStr">
@@ -35267,7 +35267,7 @@
       </c>
       <c r="R356" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S356" s="11" t="inlineStr">
@@ -38371,7 +38371,7 @@
       </c>
       <c r="R388" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S388" s="11" t="inlineStr">
@@ -41087,7 +41087,7 @@
       </c>
       <c r="R416" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S416" s="11" t="inlineStr">
@@ -42251,7 +42251,7 @@
       </c>
       <c r="R428" s="11" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S428" s="11" t="inlineStr">
@@ -46325,7 +46325,7 @@
       </c>
       <c r="R470" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S470" s="13" t="inlineStr">
@@ -47780,7 +47780,7 @@
       </c>
       <c r="R485" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S485" s="13" t="inlineStr">
@@ -53309,7 +53309,7 @@
       </c>
       <c r="R542" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S542" s="13" t="inlineStr">
@@ -53697,7 +53697,7 @@
       </c>
       <c r="R546" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S546" s="13" t="inlineStr">
@@ -54182,7 +54182,7 @@
       </c>
       <c r="R551" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S551" s="13" t="inlineStr">
@@ -54279,7 +54279,7 @@
       </c>
       <c r="R552" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S552" s="13" t="inlineStr">
@@ -54376,7 +54376,7 @@
       </c>
       <c r="R553" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S553" s="13" t="inlineStr">
@@ -58159,7 +58159,7 @@
       </c>
       <c r="R592" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S592" s="13" t="inlineStr">
@@ -60487,7 +60487,7 @@
       </c>
       <c r="R616" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S616" s="13" t="inlineStr">
@@ -61651,7 +61651,7 @@
       </c>
       <c r="R628" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S628" s="13" t="inlineStr">
@@ -62039,7 +62039,7 @@
       </c>
       <c r="R632" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S632" s="13" t="inlineStr">
@@ -62427,7 +62427,7 @@
       </c>
       <c r="R636" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S636" s="13" t="inlineStr">
@@ -62621,7 +62621,7 @@
       </c>
       <c r="R638" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S638" s="13" t="inlineStr">
@@ -63106,7 +63106,7 @@
       </c>
       <c r="R643" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S643" s="13" t="inlineStr">
@@ -65919,7 +65919,7 @@
       </c>
       <c r="R672" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S672" s="13" t="inlineStr">
@@ -66307,7 +66307,7 @@
       </c>
       <c r="R676" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S676" s="13" t="inlineStr">
@@ -72321,7 +72321,7 @@
       </c>
       <c r="R738" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S738" s="15" t="inlineStr">
@@ -73679,7 +73679,7 @@
       </c>
       <c r="R752" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S752" s="15" t="inlineStr">
@@ -73970,7 +73970,7 @@
       </c>
       <c r="R755" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S755" s="15" t="inlineStr">
@@ -74261,7 +74261,7 @@
       </c>
       <c r="R758" s="15" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S758" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Verify 13 more draft words with sources
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$770</definedName>
@@ -7234,7 +7234,7 @@
       </c>
       <c r="R67" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S67" s="7" t="inlineStr">
@@ -10241,7 +10241,7 @@
       </c>
       <c r="R98" s="7" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S98" s="7" t="inlineStr">
@@ -18389,7 +18389,7 @@
       </c>
       <c r="R182" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S182" s="9" t="inlineStr">
@@ -19553,7 +19553,7 @@
       </c>
       <c r="R194" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S194" s="9" t="inlineStr">
@@ -20135,7 +20135,7 @@
       </c>
       <c r="R200" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S200" s="9" t="inlineStr">
@@ -22075,7 +22075,7 @@
       </c>
       <c r="R220" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S220" s="9" t="inlineStr">
@@ -25179,7 +25179,7 @@
       </c>
       <c r="R252" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S252" s="9" t="inlineStr">
@@ -25373,7 +25373,7 @@
       </c>
       <c r="R254" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S254" s="9" t="inlineStr">
@@ -26052,7 +26052,7 @@
       </c>
       <c r="R261" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S261" s="9" t="inlineStr">
@@ -27313,7 +27313,7 @@
       </c>
       <c r="R274" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S274" s="9" t="inlineStr">
@@ -51369,7 +51369,7 @@
       </c>
       <c r="R522" s="13" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S522" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Verify 콘서트셋리스트 with source
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018u2EcC6iYRizzjmX4TKpRV
</commit_message>
<xml_diff>
--- a/data/kslang-slang-database.xlsx
+++ b/data/kslang-slang-database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용법 Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slang DB" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Slang DB'!$A$1:$S$770</definedName>
@@ -24694,7 +24694,7 @@
       </c>
       <c r="R247" s="9" t="inlineStr">
         <is>
-          <t>Draft — please double-check</t>
+          <t>Verified (web-checked)</t>
         </is>
       </c>
       <c r="S247" s="9" t="inlineStr">

</xml_diff>